<commit_message>
audit(pfi): clasificar hallazgos H01-H15
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="Rcffc4540d8b94fbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rdc5af93a09c848b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="Rcac61d52efc846e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="R1bdefe9af19d406b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rc690746d2f924171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="Rab323603df7f4c0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -106,28 +106,28 @@
   <x:dxfs count="4">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -433,7 +433,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Sin revisar")</x:f>
-        <x:v>67</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
         <x:v>Sin commits o pushes hacia ramas compartidas durante la auditoría.</x:v>
@@ -447,7 +447,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"En investigación")</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
         <x:v>No modificar Google Docs del tutor antes de la revisión final autorizada.</x:v>
@@ -461,7 +461,7 @@
       </x:c>
       <x:c r="B11" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Confirmado")</x:f>
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>No cambiar cifras, métricas o resultados para cerrar hallazgos.</x:v>
@@ -489,7 +489,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Ya resuelto")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
@@ -507,7 +507,7 @@
       </x:c>
       <x:c r="B15" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Bloqueado por evidencia")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -676,21 +676,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I2" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J2" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K2" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L2" s="10" t="str"/>
-      <x:c r="M2" s="10" t="str"/>
-      <x:c r="N2" s="10" t="str"/>
-      <x:c r="O2" s="10" t="str"/>
+        <x:v>Editorial</x:v>
+      </x:c>
+      <x:c r="L2" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M2" s="10" t="str">
+        <x:v>chapters/title.tex; chapters/summary.tex; chapters/abstract.tex; main.tex</x:v>
+      </x:c>
+      <x:c r="N2" s="10" t="str">
+        <x:v>main.pdf pp. 1–3: portada y datos de autor/tutor sí existen. summary.tex y abstract.tex contienen entornos vacíos y comentarios de pendiente; main.tex comenta el input de abstract. No se encontraron palabras clave.</x:v>
+      </x:c>
+      <x:c r="O2" s="10" t="str">
+        <x:v>Conservar portada; completar resumen ES/EN y palabras clave con datos y resultados verificables.</x:v>
+      </x:c>
       <x:c r="P2" s="10" t="str"/>
       <x:c r="Q2" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF actual 219 páginas; revisión final de contenido/compilación pendiente.</x:v>
       </x:c>
       <x:c r="R2" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -725,21 +733,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I3" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J3" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K3" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L3" s="10" t="str"/>
-      <x:c r="M3" s="10" t="str"/>
-      <x:c r="N3" s="10" t="str"/>
-      <x:c r="O3" s="10" t="str"/>
+        <x:v>Cierre académico</x:v>
+      </x:c>
+      <x:c r="L3" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M3" s="10" t="str">
+        <x:v>chapters/capitulo_01_introduccion.tex; chapters/capitulo_05_alcance.tex; capítulos 13–15</x:v>
+      </x:c>
+      <x:c r="N3" s="10" t="str">
+        <x:v>Introducción y alcance dicen expresamente que discusión, conclusiones y trabajos futuros permanecen pendientes; no existe capítulo general de cierre en el árbol activo.</x:v>
+      </x:c>
+      <x:c r="O3" s="10" t="str">
+        <x:v>Agregar cierre con relación objetivo → evidencia → grado de cumplimiento, discusión y límites, sin inventar resultados.</x:v>
+      </x:c>
       <x:c r="P3" s="10" t="str"/>
       <x:c r="Q3" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Diagnóstico de fuente; QA final pendiente.</x:v>
       </x:c>
       <x:c r="R3" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -774,21 +790,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I4" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Ya resuelto</x:v>
       </x:c>
       <x:c r="J4" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K4" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L4" s="10" t="str"/>
-      <x:c r="M4" s="10" t="str"/>
-      <x:c r="N4" s="10" t="str"/>
-      <x:c r="O4" s="10" t="str"/>
-      <x:c r="P4" s="10" t="str"/>
+        <x:v>Figuras y arquitectura</x:v>
+      </x:c>
+      <x:c r="L4" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M4" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_12_metodologia_validacion.tex; main.pdf</x:v>
+      </x:c>
+      <x:c r="N4" s="10" t="str">
+        <x:v>Las cuatro figuras tienen archivos y captions activos; aparecen en la lista de figuras y en main.pdf (PDF pp. 88, 90, 99, 125). Se revisó visualmente cada página: no hay marcadores de inserción.</x:v>
+      </x:c>
+      <x:c r="O4" s="10" t="str">
+        <x:v>Sin cambio en G1; conservar referencia al baseline.</x:v>
+      </x:c>
+      <x:c r="P4" s="10" t="str">
+        <x:v>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</x:v>
+      </x:c>
       <x:c r="Q4" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF actual 219 páginas; cuatro figuras renderizadas y legibles. Recompilar al cierre.</x:v>
       </x:c>
       <x:c r="R4" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -823,21 +849,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I5" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K5" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L5" s="10" t="str"/>
-      <x:c r="M5" s="10" t="str"/>
-      <x:c r="N5" s="10" t="str"/>
-      <x:c r="O5" s="10" t="str"/>
+        <x:v>Métricas y taxonomía</x:v>
+      </x:c>
+      <x:c r="L5" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M5" s="10" t="str">
+        <x:v>chapters/capitulo_11_capacidades_prototipo.tex §11.4; chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.4; appendices/anexo_e_configuracion_entrenamiento.tex</x:v>
+      </x:c>
+      <x:c r="N5" s="10" t="str">
+        <x:v>La versión actual identifica seis clases, dos fondos, raw_0 y el gate axial oficial (Dice 0,679348; IoU 0,569973), y distingue la lectura secundaria (Dice 0,810566; IoU 0,691541). La tabla de resultados no publica los seis Dice por clase.</x:v>
+      </x:c>
+      <x:c r="O5" s="10" t="str">
+        <x:v>Mantener el gate oficial y completar la tabla por clase con métricas provenientes del artifact verificable; no reinterpretar el promedio secundario como aprobado.</x:v>
+      </x:c>
       <x:c r="P5" s="10" t="str"/>
       <x:c r="Q5" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se recalcularon métricas; QA de artefacto pendiente.</x:v>
       </x:c>
       <x:c r="R5" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -872,21 +906,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I6" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K6" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L6" s="10" t="str"/>
-      <x:c r="M6" s="10" t="str"/>
-      <x:c r="N6" s="10" t="str"/>
-      <x:c r="O6" s="10" t="str"/>
+        <x:v>Alcance funcional</x:v>
+      </x:c>
+      <x:c r="L6" s="10" t="str">
+        <x:v>Gestionador LaTeX; Backend; AI Module</x:v>
+      </x:c>
+      <x:c r="M6" s="10" t="str">
+        <x:v>chapters/capitulo_05_alcance.tex §5.4; chapters/capitulo_09_requerimientos.tex RF-22; chapters/capitulo_11_capacidades_prototipo.tex §11.11.1; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N6" s="10" t="str">
+        <x:v>§5.4 excluye la clasificación degenerativa expuesta al usuario; RF-22 la llama implementada y capaz de generar ocho hallazgos; §11.11.1/Anexo F la describen bloqueada o no productiva.</x:v>
+      </x:c>
+      <x:c r="O6" s="10" t="str">
+        <x:v>Unificar como implementada en Backend/AI pero no habilitada para inferencia automática del producto; corroborar flags y rutas en los snapshots antes de corregir.</x:v>
+      </x:c>
       <x:c r="P6" s="10" t="str"/>
       <x:c r="Q6" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Contraste de código aún pendiente.</x:v>
       </x:c>
       <x:c r="R6" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -921,21 +963,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K7" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L7" s="10" t="str"/>
-      <x:c r="M7" s="10" t="str"/>
-      <x:c r="N7" s="10" t="str"/>
-      <x:c r="O7" s="10" t="str"/>
+        <x:v>Procedencia de datos y etiquetas</x:v>
+      </x:c>
+      <x:c r="L7" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M7" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.4; chapters/capitulo_11_capacidades_prototipo.tex §11.11.1; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
+      </x:c>
+      <x:c r="N7" s="10" t="str">
+        <x:v>§6.3.4 atribuye SPIDER como fuente del modelo de hallazgos por nivel; §11.11.1 identifica el clasificador de estenosis como entrenado sobre RSNA/LumbarDISC. Las fuentes y etiquetas no están trazadas por modelo en una tabla única.</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="str">
+        <x:v>Separar dataset, tarea, clases/etiquetas y partición por modelo; verificar los manifests antes de completar números.</x:v>
+      </x:c>
       <x:c r="P7" s="10" t="str"/>
       <x:c r="Q7" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se ejecutó entrenamiento ni se reconstruyeron particiones.</x:v>
       </x:c>
       <x:c r="R7" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -970,21 +1020,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I8" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K8" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L8" s="10" t="str"/>
-      <x:c r="M8" s="10" t="str"/>
-      <x:c r="N8" s="10" t="str"/>
-      <x:c r="O8" s="10" t="str"/>
+        <x:v>E2E y evidencia QA</x:v>
+      </x:c>
+      <x:c r="L8" s="10" t="str">
+        <x:v>Gestionador LaTeX; Backend; Frontend; AI Module</x:v>
+      </x:c>
+      <x:c r="M8" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.8; appendices/anexo_a_cronograma.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N8" s="10" t="str">
+        <x:v>§13.8 registra Playwright 11/11 para recorrido demo/funcional; Anexo A mantiene dos filas para E2E con estados distintos (una cerrada y otra parcial). Falta cotejar logs/runner y el alcance exacto del Full Product UI.</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="str">
+        <x:v>Reconciliar la fila duplicada y enlazar evidencia de runner por alcance: demo, stack local y Cloud V2.</x:v>
+      </x:c>
       <x:c r="P8" s="10" t="str"/>
       <x:c r="Q8" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>La evidencia automatizada no fue ejecutada en esta pasada.</x:v>
       </x:c>
       <x:c r="R8" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1019,21 +1077,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I9" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K9" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L9" s="10" t="str"/>
-      <x:c r="M9" s="10" t="str"/>
-      <x:c r="N9" s="10" t="str"/>
-      <x:c r="O9" s="10" t="str"/>
+        <x:v>Hitos y estados</x:v>
+      </x:c>
+      <x:c r="L9" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="str">
+        <x:v>chapters/capitulo_05_alcance.tex §5.6; chapters/capitulo_14_planificacion_academica.tex; appendices/anexo_a_cronograma.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N9" s="10" t="str">
+        <x:v>El documento mantiene tareas futuras (entrega del 75 %, validación profesional final y conclusiones); no se encontró una afirmación explícita “100 %” en el texto activo/PDF consultado. Falta reconciliar el hito al que refiere el hallazgo.</x:v>
+      </x:c>
+      <x:c r="O9" s="10" t="str">
+        <x:v>Definir fecha de corte y distinguir entrega académica, cierre de software y actividades posteriores.</x:v>
+      </x:c>
       <x:c r="P9" s="10" t="str"/>
       <x:c r="Q9" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Pendiente cotejar estados de Tablas 13.5/H.1 y Google Docs, sin editarlo.</x:v>
       </x:c>
       <x:c r="R9" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1068,21 +1134,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I10" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K10" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L10" s="10" t="str"/>
-      <x:c r="M10" s="10" t="str"/>
-      <x:c r="N10" s="10" t="str"/>
-      <x:c r="O10" s="10" t="str"/>
+        <x:v>Identidad longitudinal</x:v>
+      </x:c>
+      <x:c r="L10" s="10" t="str">
+        <x:v>Gestionador LaTeX; Backend; Frontend</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="str">
+        <x:v>chapters/capitulo_05_alcance.tex §5.5; chapters/capitulo_09_requerimientos.tex RF-08/RF-14; chapters/capitulo_11_capacidades_prototipo.tex §§11.1, 11.9; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
+      </x:c>
+      <x:c r="N10" s="10" t="str">
+        <x:v>La fuente distingue Patient/patientId como dominio persistido en Backend y subjectRef como compatibilidad usada por historial/longitudinal en Frontend Demo. Debe verificarse el contrato y el comportamiento en snapshots para saber si RF-08 describe estado o intención.</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="str">
+        <x:v>Mantener explícita la separación API/Frontend y ajustar estados de requisito a la evidencia de integración.</x:v>
+      </x:c>
       <x:c r="P10" s="10" t="str"/>
       <x:c r="Q10" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Revisión de código de los tres repositorios pendiente.</x:v>
       </x:c>
       <x:c r="R10" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1117,21 +1191,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I11" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K11" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L11" s="10" t="str"/>
-      <x:c r="M11" s="10" t="str"/>
-      <x:c r="N11" s="10" t="str"/>
-      <x:c r="O11" s="10" t="str"/>
+        <x:v>Alcance y capacidades</x:v>
+      </x:c>
+      <x:c r="L11" s="10" t="str">
+        <x:v>Gestionador LaTeX; Backend; Frontend; AI Module</x:v>
+      </x:c>
+      <x:c r="M11" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex; chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_11_capacidades_prototipo.tex; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
+      </x:c>
+      <x:c r="N11" s="10" t="str">
+        <x:v>El capítulo 11 documenta Demo Mode, exportación PDF/JSON, Grad-CAM experimental, 67B2/67C y chat mock/Qwen como capacidades con estados diferenciados. Falta revisar trazabilidad formal a alcance/RF y la frase de exclusión de LLM.</x:v>
+      </x:c>
+      <x:c r="O11" s="10" t="str">
+        <x:v>Cruzar cada elemento con alcance, RF y código; resolver solo los casos sin definición/estado consistente.</x:v>
+      </x:c>
       <x:c r="P11" s="10" t="str"/>
       <x:c r="Q11" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se modificó el alcance ni se verificó proveedor productivo.</x:v>
       </x:c>
       <x:c r="R11" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1166,21 +1248,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K12" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L12" s="10" t="str"/>
-      <x:c r="M12" s="10" t="str"/>
-      <x:c r="N12" s="10" t="str"/>
-      <x:c r="O12" s="10" t="str"/>
+        <x:v>Metodología de evaluación axial</x:v>
+      </x:c>
+      <x:c r="L12" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M12" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.2; chapters/capitulo_11_capacidades_prototipo.tex §11.4; artifacts/manifests y cuaderno axial por localizar</x:v>
+      </x:c>
+      <x:c r="N12" s="10" t="str">
+        <x:v>La tabla consigna entrenamiento “Pendiente de recuperación”, 81 casos de validación y 102 de prueba; el texto admite dos particiones axiales no coincidentes y ausencia de conteos definitivos. No hay evidencia suficiente para reconstruirlos sin el manifest/cuaderno correcto.</x:v>
+      </x:c>
+      <x:c r="O12" s="10" t="str">
+        <x:v>Solicitar/localizar el manifest y el cuaderno exactos; documentar partición por paciente. No reentrenar ni inventar conteos.</x:v>
+      </x:c>
       <x:c r="P12" s="10" t="str"/>
       <x:c r="Q12" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se ejecutó entrenamiento ni evaluación.</x:v>
       </x:c>
       <x:c r="R12" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1215,21 +1305,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I13" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K13" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L13" s="10" t="str"/>
-      <x:c r="M13" s="10" t="str"/>
-      <x:c r="N13" s="10" t="str"/>
-      <x:c r="O13" s="10" t="str"/>
+        <x:v>Métricas y criterio de promoción</x:v>
+      </x:c>
+      <x:c r="L13" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M13" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.4; chapters/capitulo_07_marco_teorico.tex §7.9</x:v>
+      </x:c>
+      <x:c r="N13" s="10" t="str">
+        <x:v>El protocolo vigente exige IoU como condición; tabla de resultados informa IoU axial pero no para SPIDER sagital. HD95/NSD se explican teóricamente y no se reportan resultados.</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="str">
+        <x:v>Recuperar IoU por modelo y reportarlo; si HD95 no existe, declararlo no calculado y revisar que el objetivo/criterio no prometa esa evidencia.</x:v>
+      </x:c>
       <x:c r="P13" s="10" t="str"/>
       <x:c r="Q13" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Datos de evaluación fuente pendientes; no se recalcularon métricas.</x:v>
       </x:c>
       <x:c r="R13" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1264,21 +1362,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I14" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K14" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L14" s="10" t="str"/>
-      <x:c r="M14" s="10" t="str"/>
-      <x:c r="N14" s="10" t="str"/>
-      <x:c r="O14" s="10" t="str"/>
+        <x:v>Modelo económico</x:v>
+      </x:c>
+      <x:c r="L14" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M14" s="10" t="str">
+        <x:v>chapters/capitulo_15_modelo_negocio.tex; financial/MIRA_L_Modelo_Financiero_36M_Reconciliado_2026_con_payback_dinamico.xlsx; financial/PFI_RM_LUMBAR_FINANCIAL_MODEL_36M.xlsx</x:v>
+      </x:c>
+      <x:c r="N14" s="10" t="str">
+        <x:v>La tesis y el repositorio sí contienen hojas de cálculo; el texto explica escenarios/supuestos y declara que adquisición, churn, volumen y disposición a pagar no son observados. La reproducibilidad y valores fraccionarios (13,41 clientes) requieren inspección del libro canónico.</x:v>
+      </x:c>
+      <x:c r="O14" s="10" t="str">
+        <x:v>Inspeccionar fórmulas, selector, supuestos y reconciliación con las tablas de tesis; diferenciar salidas fraccionarias esperadas de conteos observados.</x:v>
+      </x:c>
       <x:c r="P14" s="10" t="str"/>
       <x:c r="Q14" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se alteró ni recalculó el modelo financiero.</x:v>
       </x:c>
       <x:c r="R14" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1313,21 +1419,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I15" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K15" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L15" s="10" t="str"/>
-      <x:c r="M15" s="10" t="str"/>
-      <x:c r="N15" s="10" t="str"/>
-      <x:c r="O15" s="10" t="str"/>
+        <x:v>Validación profesional y ética</x:v>
+      </x:c>
+      <x:c r="L15" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M15" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex; chapters/capitulo_13_resultados_evaluacion.tex §13.11; appendices/anexo_d_entrevistas.tex; appendices/anexo_h_validacion_profesional.tex</x:v>
+      </x:c>
+      <x:c r="N15" s="10" t="str">
+        <x:v>El PDF describe dos sesiones y sus aportes; las transcripciones del Anexo D no muestran fecha en los fragmentos revisados. La existencia de consentimientos, registros de sesión y autorizaciones no está demostrada por la fuente citada.</x:v>
+      </x:c>
+      <x:c r="O15" s="10" t="str">
+        <x:v>Verificar anexos/archivos de respaldo y limitar afirmaciones al registro disponible; no recrear fechas, consentimiento ni grabaciones.</x:v>
+      </x:c>
       <x:c r="P15" s="10" t="str"/>
       <x:c r="Q15" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>Pendiente localizar registros; no se contactó a profesionales.</x:v>
       </x:c>
       <x:c r="R15" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1362,21 +1476,29 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I16" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K16" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L16" s="10" t="str"/>
-      <x:c r="M16" s="10" t="str"/>
-      <x:c r="N16" s="10" t="str"/>
-      <x:c r="O16" s="10" t="str"/>
+        <x:v>QA de software</x:v>
+      </x:c>
+      <x:c r="L16" s="10" t="str">
+        <x:v>Gestionador LaTeX; Backend; AI Module</x:v>
+      </x:c>
+      <x:c r="M16" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.8; reportes de pruebas en repositorios Backend/AI</x:v>
+      </x:c>
+      <x:c r="N16" s="10" t="str">
+        <x:v>La tabla de pruebas declara AI full suite 479 passed / 40 failed y explica que no es totalmente verde; la observación del tutor sobre fallos persistentes no queda resuelta por esa declaración. Los 78 del Backend requieren cotejo de reporte.</x:v>
+      </x:c>
+      <x:c r="O16" s="10" t="str">
+        <x:v>Reproducir el comando/documento de suite; identificar cada fallo y si es ambiental, aislarlo con skip condicionado y razón, o reparar sin esconder fallos.</x:v>
+      </x:c>
       <x:c r="P16" s="10" t="str"/>
       <x:c r="Q16" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>No se ejecutaron suites en G1.</x:v>
       </x:c>
       <x:c r="R16" s="10" t="str">
         <x:v>No revisado</x:v>

</xml_diff>

<commit_message>
audit(pfi): record G3 status and verification evidence
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="R1bdefe9af19d406b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rc690746d2f924171"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="Rab323603df7f4c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="Rfccff9b7e80c4f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rfb497684af094cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="R624eb0ce88804e70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -433,7 +433,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Sin revisar")</x:f>
-        <x:v>52</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
         <x:v>Sin commits o pushes hacia ramas compartidas durante la auditoría.</x:v>
@@ -447,7 +447,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"En investigación")</x:f>
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
         <x:v>No modificar Google Docs del tutor antes de la revisión final autorizada.</x:v>
@@ -461,7 +461,7 @@
       </x:c>
       <x:c r="B11" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Confirmado")</x:f>
-        <x:v>7</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>No cambiar cifras, métricas o resultados para cerrar hallazgos.</x:v>
@@ -475,7 +475,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Corrección aplicada")</x:f>
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
         <x:v>No cerrar si faltan evidencias técnicas o pruebas exigidas.</x:v>
@@ -489,7 +489,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Ya resuelto")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
@@ -507,7 +507,7 @@
       </x:c>
       <x:c r="B15" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Bloqueado por evidencia")</x:f>
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -516,7 +516,7 @@
       </x:c>
       <x:c r="B16" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Cerrado con evidencia")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
@@ -525,7 +525,7 @@
       </x:c>
       <x:c r="B17" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!S2:S68,"QA aprobado")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
@@ -676,7 +676,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I2" s="10" t="str">
-        <x:v>Confirmado</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J2" s="10" t="str">
         <x:v>Parcial</x:v>
@@ -694,11 +694,13 @@
         <x:v>main.pdf pp. 1–3: portada y datos de autor/tutor sí existen. summary.tex y abstract.tex contienen entornos vacíos y comentarios de pendiente; main.tex comenta el input de abstract. No se encontraron palabras clave.</x:v>
       </x:c>
       <x:c r="O2" s="10" t="str">
-        <x:v>Conservar portada; completar resumen ES/EN y palabras clave con datos y resultados verificables.</x:v>
-      </x:c>
-      <x:c r="P2" s="10" t="str"/>
+        <x:v>Se conservó la portada existente y se completaron el resumen y abstract bilingües con palabras clave y resultados respaldados.</x:v>
+      </x:c>
+      <x:c r="P2" s="10" t="str">
+        <x:v>58e29fcb34942a7cf3107908f1f4911791df70d4</x:v>
+      </x:c>
       <x:c r="Q2" s="10" t="str">
-        <x:v>PDF actual 219 páginas; revisión final de contenido/compilación pendiente.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R2" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -733,7 +735,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I3" s="10" t="str">
-        <x:v>Confirmado</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J3" s="10" t="str">
         <x:v>Sí</x:v>
@@ -751,11 +753,13 @@
         <x:v>Introducción y alcance dicen expresamente que discusión, conclusiones y trabajos futuros permanecen pendientes; no existe capítulo general de cierre en el árbol activo.</x:v>
       </x:c>
       <x:c r="O3" s="10" t="str">
-        <x:v>Agregar cierre con relación objetivo → evidencia → grado de cumplimiento, discusión y límites, sin inventar resultados.</x:v>
-      </x:c>
-      <x:c r="P3" s="10" t="str"/>
+        <x:v>Se agregó un capítulo final con relación objetivo–evidencia–cumplimiento, discusión, limitaciones y trabajo futuro; la redacción conserva los límites reales de la evidencia.</x:v>
+      </x:c>
+      <x:c r="P3" s="10" t="str">
+        <x:v>58e29fcb34942a7cf3107908f1f4911791df70d4</x:v>
+      </x:c>
       <x:c r="Q3" s="10" t="str">
-        <x:v>Diagnóstico de fuente; QA final pendiente.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R3" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -790,7 +794,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I4" s="10" t="str">
-        <x:v>Ya resuelto</x:v>
+        <x:v>Cerrado con evidencia</x:v>
       </x:c>
       <x:c r="J4" s="10" t="str">
         <x:v>No</x:v>
@@ -808,18 +812,20 @@
         <x:v>Las cuatro figuras tienen archivos y captions activos; aparecen en la lista de figuras y en main.pdf (PDF pp. 88, 90, 99, 125). Se revisó visualmente cada página: no hay marcadores de inserción.</x:v>
       </x:c>
       <x:c r="O4" s="10" t="str">
-        <x:v>Sin cambio en G1; conservar referencia al baseline.</x:v>
+        <x:v>Cerrado con evidencia: las cuatro figuras cuestionadas aparecen en el PDF final con diagramas/captions activos y se revisaron visualmente las páginas físicas 93, 95, 104 y 131.</x:v>
       </x:c>
       <x:c r="P4" s="10" t="str">
         <x:v>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</x:v>
       </x:c>
       <x:c r="Q4" s="10" t="str">
-        <x:v>PDF actual 219 páginas; cuatro figuras renderizadas y legibles. Recompilar al cierre.</x:v>
+        <x:v>PDF final 231 páginas; figuras activas y referencias cruzadas verificadas mediante extracción y revisión visual de páginas representativas.</x:v>
       </x:c>
       <x:c r="R4" s="10" t="str">
         <x:v>No revisado</x:v>
       </x:c>
-      <x:c r="S4" s="10" t="str"/>
+      <x:c r="S4" s="10" t="str">
+        <x:v>QA aprobado</x:v>
+      </x:c>
       <x:c r="T4" s="10" t="str"/>
       <x:c r="U4" s="10" t="str"/>
     </x:row>
@@ -906,7 +912,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I6" s="10" t="str">
-        <x:v>Confirmado</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
         <x:v>Sí</x:v>
@@ -921,14 +927,16 @@
         <x:v>chapters/capitulo_05_alcance.tex §5.4; chapters/capitulo_09_requerimientos.tex RF-22; chapters/capitulo_11_capacidades_prototipo.tex §11.11.1; appendices/anexo_f_evolucion_tecnica.tex</x:v>
       </x:c>
       <x:c r="N6" s="10" t="str">
-        <x:v>§5.4 excluye la clasificación degenerativa expuesta al usuario; RF-22 la llama implementada y capaz de generar ocho hallazgos; §11.11.1/Anexo F la describen bloqueada o no productiva.</x:v>
+        <x:v>RF-22 contempla ocho categorías P10.7, pero la ruta de producto permanece bloqueada por blocked_preprocessing_parity y automaticInferenceEnabled=false; la tesis documenta la distinción entre implementación contractual y disponibilidad de inferencia automática. Snapshots locales de Backend y AI contrastados; no se modificó código de producto.</x:v>
       </x:c>
       <x:c r="O6" s="10" t="str">
-        <x:v>Unificar como implementada en Backend/AI pero no habilitada para inferencia automática del producto; corroborar flags y rutas en los snapshots antes de corregir.</x:v>
-      </x:c>
-      <x:c r="P6" s="10" t="str"/>
+        <x:v>Se aclaró que RF-22 define las ocho categorías P10.7 pero la inferencia automática del producto está deshabilitada por blocked_preprocessing_parity y automaticInferenceEnabled=false; sin cambios de código.</x:v>
+      </x:c>
+      <x:c r="P6" s="10" t="str">
+        <x:v>21295af8462380cf1591ca607c1aad7cbe708b0a</x:v>
+      </x:c>
       <x:c r="Q6" s="10" t="str">
-        <x:v>Contraste de código aún pendiente.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R6" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -963,7 +971,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
-        <x:v>Confirmado</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
         <x:v>Sí</x:v>
@@ -978,14 +986,16 @@
         <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.4; chapters/capitulo_11_capacidades_prototipo.tex §11.11.1; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
       </x:c>
       <x:c r="N7" s="10" t="str">
-        <x:v>§6.3.4 atribuye SPIDER como fuente del modelo de hallazgos por nivel; §11.11.1 identifica el clasificador de estenosis como entrenado sobre RSNA/LumbarDISC. Las fuentes y etiquetas no están trazadas por modelo en una tabla única.</x:v>
+        <x:v>P10.6: clasificación axial de estenosis subarticular con RSNA/LumbarDISC. P10.7: estimación de ocho hallazgos sagitales con SPIDER. La tesis ahora separa tarea, dataset y alcance; no se afirma reconstrucción de particiones ni reentrenamiento.</x:v>
       </x:c>
       <x:c r="O7" s="10" t="str">
-        <x:v>Separar dataset, tarea, clases/etiquetas y partición por modelo; verificar los manifests antes de completar números.</x:v>
-      </x:c>
-      <x:c r="P7" s="10" t="str"/>
+        <x:v>Se separaron P10.6 (clasificador axial RSNA/LumbarDISC) y P10.7 (ocho hallazgos sagitales SPIDER); se documentó tarea y procedencia sin reconstruir particiones ni reentrenar.</x:v>
+      </x:c>
+      <x:c r="P7" s="10" t="str">
+        <x:v>4f27a62214e254e1d991cba379b4c9c6cbf5d52b</x:v>
+      </x:c>
       <x:c r="Q7" s="10" t="str">
-        <x:v>No se ejecutó entrenamiento ni se reconstruyeron particiones.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R7" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1020,29 +1030,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I8" s="10" t="str">
-        <x:v>En investigación</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K8" s="10" t="str">
         <x:v>E2E y evidencia QA</x:v>
       </x:c>
       <x:c r="L8" s="10" t="str">
-        <x:v>Gestionador LaTeX; Backend; Frontend; AI Module</x:v>
+        <x:v>Gestionador LaTeX; Frontend; Backend</x:v>
       </x:c>
       <x:c r="M8" s="10" t="str">
-        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.8; appendices/anexo_a_cronograma.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §§13.8–13.9; chapters/capitulo_11_capacidades_prototipo.tex; chapters/capitulo_14_planificacion_academica.tex; appendices/anexo_a_cronograma.tex; appendices/anexo_f_evolucion_tecnica.tex; Frontend docs/post_e50/87_BROWSER_FULL_FLOW.md; Backend docs/post_e50/87_FULL_DOCKER_E2E.md</x:v>
       </x:c>
       <x:c r="N8" s="10" t="str">
-        <x:v>§13.8 registra Playwright 11/11 para recorrido demo/funcional; Anexo A mantiene dos filas para E2E con estados distintos (una cerrada y otra parcial). Falta cotejar logs/runner y el alcance exacto del Full Product UI.</x:v>
+        <x:v>Los reports Stage 87 describen el flujo principal Browser E2E aprobado en tres ejecuciones con bytes sintéticos y mock de IA; selector de corrección/chat parcialmente automatizados y comprobados por API. Se retiró la fila duplicada y se diferenciaron resultado acotado y cierre global parcial.</x:v>
       </x:c>
       <x:c r="O8" s="10" t="str">
-        <x:v>Reconciliar la fila duplicada y enlazar evidencia de runner por alcance: demo, stack local y Cloud V2.</x:v>
-      </x:c>
-      <x:c r="P8" s="10" t="str"/>
+        <x:v>Precisar alcances; no atribuir 11/11 al flujo global.</x:v>
+      </x:c>
+      <x:c r="P8" s="10" t="str">
+        <x:v>304153cbdbc0a1908efa9d361d03bbe148d30a92</x:v>
+      </x:c>
       <x:c r="Q8" s="10" t="str">
-        <x:v>La evidencia automatizada no fue ejecutada en esta pasada.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R8" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1077,7 +1089,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I9" s="10" t="str">
-        <x:v>En investigación</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
         <x:v>Parcial</x:v>
@@ -1092,14 +1104,16 @@
         <x:v>chapters/capitulo_05_alcance.tex §5.6; chapters/capitulo_14_planificacion_academica.tex; appendices/anexo_a_cronograma.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
       </x:c>
       <x:c r="N9" s="10" t="str">
-        <x:v>El documento mantiene tareas futuras (entrega del 75 %, validación profesional final y conclusiones); no se encontró una afirmación explícita “100 %” en el texto activo/PDF consultado. Falta reconciliar el hito al que refiere el hallazgo.</x:v>
+        <x:v>La planificación se reconcilió con la entrega académica del 75 % y la defensa, distinguiéndolas del cierre de software y la validación profesional posterior. No se editó Google Docs; queda pendiente confirmar el estado de hitos externos.</x:v>
       </x:c>
       <x:c r="O9" s="10" t="str">
-        <x:v>Definir fecha de corte y distinguir entrega académica, cierre de software y actividades posteriores.</x:v>
-      </x:c>
-      <x:c r="P9" s="10" t="str"/>
+        <x:v>Se alineó el cronograma académico con la entrega del 75 % y la defensa, separándolos del cierre de software y la validación profesional posterior.</x:v>
+      </x:c>
+      <x:c r="P9" s="10" t="str">
+        <x:v>ecaf4cf6e4c57bb08f506167b430ca7b8289feb6</x:v>
+      </x:c>
       <x:c r="Q9" s="10" t="str">
-        <x:v>Pendiente cotejar estados de Tablas 13.5/H.1 y Google Docs, sin editarlo.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R9" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1248,7 +1262,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
-        <x:v>Bloqueado por evidencia</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
         <x:v>Sí</x:v>
@@ -1263,14 +1277,16 @@
         <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.2; chapters/capitulo_11_capacidades_prototipo.tex §11.4; artifacts/manifests y cuaderno axial por localizar</x:v>
       </x:c>
       <x:c r="N12" s="10" t="str">
-        <x:v>La tabla consigna entrenamiento “Pendiente de recuperación”, 81 casos de validación y 102 de prueba; el texto admite dos particiones axiales no coincidentes y ausencia de conteos definitivos. No hay evidencia suficiente para reconstruirlos sin el manifest/cuaderno correcto.</x:v>
+        <x:v>E9: ZIP de informe anonimizado y manifiesto SHA-256 preservados en evidencias locales; 610 registros (427/81/102), 184 IDs de paciente sin intersecciones, sin filas idénticas. Persisten la diferencia con el split histórico no aportado, reutilización previa del test, duplicados por contenido no comprobados y rutas de máscara repetidas.</x:v>
       </x:c>
       <x:c r="O12" s="10" t="str">
-        <x:v>Solicitar/localizar el manifest y el cuaderno exactos; documentar partición por paciente. No reentrenar ni inventar conteos.</x:v>
-      </x:c>
-      <x:c r="P12" s="10" t="str"/>
+        <x:v>Se incorporaron los conteos y trazas verificables del split E9, junto con los límites de uso previo del test, falta del split histórico alternativo y ausencia de control de duplicados por contenido. Resolución parcial.</x:v>
+      </x:c>
+      <x:c r="P12" s="10" t="str">
+        <x:v>461cd1a5a7efed8840f7008116e713208cda125a</x:v>
+      </x:c>
       <x:c r="Q12" s="10" t="str">
-        <x:v>No se ejecutó entrenamiento ni evaluación.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R12" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1362,7 +1378,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I14" s="10" t="str">
-        <x:v>En investigación</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
         <x:v>Parcial</x:v>
@@ -1377,14 +1393,16 @@
         <x:v>chapters/capitulo_15_modelo_negocio.tex; financial/MIRA_L_Modelo_Financiero_36M_Reconciliado_2026_con_payback_dinamico.xlsx; financial/PFI_RM_LUMBAR_FINANCIAL_MODEL_36M.xlsx</x:v>
       </x:c>
       <x:c r="N14" s="10" t="str">
-        <x:v>La tesis y el repositorio sí contienen hojas de cálculo; el texto explica escenarios/supuestos y declara que adquisición, churn, volumen y disposición a pagar no son observados. La reproducibilidad y valores fraccionarios (13,41 clientes) requieren inspección del libro canónico.</x:v>
+        <x:v>El libro canónico reconciliado MIRA_L_Modelo_Financiero_36M_Reconciliado_2026_con_payback_dinamico.xlsx fue inspeccionado: supuestos/fórmulas en 01_SUPUESTOS y 04_BASE, resultados en 02_RESULTADOS. Se incorporó una tabla de entradas y una aclaración de que 13,41 clientes son equivalentes esperados matemáticos, no instituciones observadas. No hay ventas, clientes ni adquisición observada.</x:v>
       </x:c>
       <x:c r="O14" s="10" t="str">
-        <x:v>Inspeccionar fórmulas, selector, supuestos y reconciliación con las tablas de tesis; diferenciar salidas fraccionarias esperadas de conteos observados.</x:v>
-      </x:c>
-      <x:c r="P14" s="10" t="str"/>
+        <x:v>Se transcribieron los supuestos verificados del libro canónico y se aclaró que los clientes fraccionarios son equivalentes esperados del modelo, no observaciones comerciales.</x:v>
+      </x:c>
+      <x:c r="P14" s="10" t="str">
+        <x:v>643e657502440e933c59f1356e3beae1edd5df44</x:v>
+      </x:c>
       <x:c r="Q14" s="10" t="str">
-        <x:v>No se alteró ni recalculó el modelo financiero.</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R14" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1419,7 +1437,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I15" s="10" t="str">
-        <x:v>En investigación</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
         <x:v>Parcial</x:v>
@@ -1434,14 +1452,14 @@
         <x:v>chapters/capitulo_08_user_research.tex; chapters/capitulo_13_resultados_evaluacion.tex §13.11; appendices/anexo_d_entrevistas.tex; appendices/anexo_h_validacion_profesional.tex</x:v>
       </x:c>
       <x:c r="N15" s="10" t="str">
-        <x:v>El PDF describe dos sesiones y sus aportes; las transcripciones del Anexo D no muestran fecha en los fragmentos revisados. La existencia de consentimientos, registros de sesión y autorizaciones no está demostrada por la fuente citada.</x:v>
+        <x:v>Las descripciones de sesiones carecen de fechas verificables y el expediente disponible no acredita consentimientos ni autorizaciones para publicación. Se limita la redacción a las fuentes disponibles; no se recrearon metadatos.</x:v>
       </x:c>
       <x:c r="O15" s="10" t="str">
-        <x:v>Verificar anexos/archivos de respaldo y limitar afirmaciones al registro disponible; no recrear fechas, consentimiento ni grabaciones.</x:v>
+        <x:v>Bloqueado hasta localizar registros fechados de sesiones, consentimientos y autorizaciones; no se inventaron metadatos ni se contactó a los profesionales.</x:v>
       </x:c>
       <x:c r="P15" s="10" t="str"/>
       <x:c r="Q15" s="10" t="str">
-        <x:v>Pendiente localizar registros; no se contactó a profesionales.</x:v>
+        <x:v>Bloqueado: faltan registros de sesiones fechados, consentimientos y autorizaciones; requiere evidencia documental externa al repositorio.</x:v>
       </x:c>
       <x:c r="R15" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -1533,26 +1551,38 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I17" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Cerrado con evidencia</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K17" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L17" s="10" t="str"/>
-      <x:c r="M17" s="10" t="str"/>
-      <x:c r="N17" s="10" t="str"/>
-      <x:c r="O17" s="10" t="str"/>
-      <x:c r="P17" s="10" t="str"/>
+        <x:v>Revisión editorial</x:v>
+      </x:c>
+      <x:c r="L17" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M17" s="10" t="str">
+        <x:v>chapters/capitulo_01_introduccion.tex</x:v>
+      </x:c>
+      <x:c r="N17" s="10" t="str">
+        <x:v>El capítulo contiene un solo párrafo de organización documental; la duplicación citada no se reproduce en el fuente actual.</x:v>
+      </x:c>
+      <x:c r="O17" s="10" t="str">
+        <x:v>Cerrado con evidencia: la duplicación no aparece en el PDF final y el párrafo de organización documental aparece una sola vez en la página física 19.</x:v>
+      </x:c>
+      <x:c r="P17" s="10" t="str">
+        <x:v>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</x:v>
+      </x:c>
       <x:c r="Q17" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R17" s="10" t="str">
         <x:v>No revisado</x:v>
       </x:c>
-      <x:c r="S17" s="10" t="str"/>
+      <x:c r="S17" s="10" t="str">
+        <x:v>QA aprobado</x:v>
+      </x:c>
       <x:c r="T17" s="10" t="str"/>
       <x:c r="U17" s="10" t="str"/>
     </x:row>
@@ -1582,26 +1612,38 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I18" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Cerrado con evidencia</x:v>
       </x:c>
       <x:c r="J18" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K18" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L18" s="10" t="str"/>
-      <x:c r="M18" s="10" t="str"/>
-      <x:c r="N18" s="10" t="str"/>
-      <x:c r="O18" s="10" t="str"/>
-      <x:c r="P18" s="10" t="str"/>
+        <x:v>Revisión editorial</x:v>
+      </x:c>
+      <x:c r="L18" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M18" s="10" t="str">
+        <x:v>chapters/capitulo_05_alcance.tex §5.6</x:v>
+      </x:c>
+      <x:c r="N18" s="10" t="str">
+        <x:v>Existe el encabezado “Alcance del documento final” con un único párrafo; las dos frases citadas no aparecen en el fuente actual.</x:v>
+      </x:c>
+      <x:c r="O18" s="10" t="str">
+        <x:v>Cerrado con evidencia: el encabezado 5.6 “Alcance del documento final” figura en el índice y en la página física 25; las dos frases duplicadas no aparecen en el PDF final.</x:v>
+      </x:c>
+      <x:c r="P18" s="10" t="str">
+        <x:v>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</x:v>
+      </x:c>
       <x:c r="Q18" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R18" s="10" t="str">
         <x:v>No revisado</x:v>
       </x:c>
-      <x:c r="S18" s="10" t="str"/>
+      <x:c r="S18" s="10" t="str">
+        <x:v>QA aprobado</x:v>
+      </x:c>
       <x:c r="T18" s="10" t="str"/>
       <x:c r="U18" s="10" t="str"/>
     </x:row>
@@ -1631,18 +1673,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I19" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J19" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K19" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L19" s="10" t="str"/>
-      <x:c r="M19" s="10" t="str"/>
-      <x:c r="N19" s="10" t="str"/>
-      <x:c r="O19" s="10" t="str"/>
+        <x:v>Edición científica/documental</x:v>
+      </x:c>
+      <x:c r="L19" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M19" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §§6.3.3–6.3.4; appendices/anexo_c_modulo_axial_preliminar.tex</x:v>
+      </x:c>
+      <x:c r="N19" s="10" t="str">
+        <x:v>La descripción de población, secuencias y anotadores aparece en cuerpo y anexo; hay repetición parcial de especificaciones y cifras.</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="str">
+        <x:v>Conservar una descripción principal y referenciarla desde el anexo, después de verificar los conteos en la fuente primaria.</x:v>
+      </x:c>
       <x:c r="P19" s="10" t="str"/>
       <x:c r="Q19" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1680,18 +1730,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I20" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J20" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K20" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L20" s="10" t="str"/>
-      <x:c r="M20" s="10" t="str"/>
-      <x:c r="N20" s="10" t="str"/>
-      <x:c r="O20" s="10" t="str"/>
+        <x:v>Edición de resultados</x:v>
+      </x:c>
+      <x:c r="L20" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M20" s="10" t="str">
+        <x:v>chapters/capitulo_11_capacidades_prototipo.tex §11.5; chapters/capitulo_13_resultados_evaluacion.tex §§13.4–13.6</x:v>
+      </x:c>
+      <x:c r="N20" s="10" t="str">
+        <x:v>La falta de validación profesional de mediciones y el contraste con rangos se reiteran en capacidades, resultados y limitaciones.</x:v>
+      </x:c>
+      <x:c r="O20" s="10" t="str">
+        <x:v>Dejar explicación completa en resultados y usar referencias breves en capacidades/limitaciones.</x:v>
+      </x:c>
       <x:c r="P20" s="10" t="str"/>
       <x:c r="Q20" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1729,18 +1787,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I21" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J21" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K21" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L21" s="10" t="str"/>
-      <x:c r="M21" s="10" t="str"/>
-      <x:c r="N21" s="10" t="str"/>
-      <x:c r="O21" s="10" t="str"/>
+        <x:v>Edición de resultados</x:v>
+      </x:c>
+      <x:c r="L21" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M21" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.12</x:v>
+      </x:c>
+      <x:c r="N21" s="10" t="str">
+        <x:v>El cierre enumera límites que también se desarrollan por separado; hay solapamiento en partición axial, métricas y validación independiente.</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="str">
+        <x:v>Consolidar sin eliminar límites distintos ni reducir una limitación con impacto metodológico.</x:v>
+      </x:c>
       <x:c r="P21" s="10" t="str"/>
       <x:c r="Q21" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1778,18 +1844,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I22" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J22" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K22" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L22" s="10" t="str"/>
-      <x:c r="M22" s="10" t="str"/>
-      <x:c r="N22" s="10" t="str"/>
-      <x:c r="O22" s="10" t="str"/>
+        <x:v>Edición de modelo financiero</x:v>
+      </x:c>
+      <x:c r="L22" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M22" s="10" t="str">
+        <x:v>chapters/capitulo_15_modelo_negocio.tex §§14.14–14.15 según índice fuente</x:v>
+      </x:c>
+      <x:c r="N22" s="10" t="str">
+        <x:v>El hallazgo describe numeración y párrafos repetidos en el cierre financiero; requiere corregir lista y dejar una síntesis única.</x:v>
+      </x:c>
+      <x:c r="O22" s="10" t="str">
+        <x:v>Revisar ítems contra el texto antes de renumerar; conservar conclusiones numéricas verificadas.</x:v>
+      </x:c>
       <x:c r="P22" s="10" t="str"/>
       <x:c r="Q22" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1827,18 +1901,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I23" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J23" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K23" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L23" s="10" t="str"/>
-      <x:c r="M23" s="10" t="str"/>
-      <x:c r="N23" s="10" t="str"/>
-      <x:c r="O23" s="10" t="str"/>
+        <x:v>Edición de arquitectura Cloud</x:v>
+      </x:c>
+      <x:c r="L23" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M23" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §§10.7.1–10.7.3; chapters/capitulo_12_metodologia_validacion.tex; chapters/capitulo_13_resultados_evaluacion.tex §13.9</x:v>
+      </x:c>
+      <x:c r="N23" s="10" t="str">
+        <x:v>V1/V2, la observación de RUNNABLE/ALWAYS y pausa/restauración V1 vuelven en varios lugares; parte de la repetición aclara alcances distintos.</x:v>
+      </x:c>
+      <x:c r="O23" s="10" t="str">
+        <x:v>Mantener una explicación canónica V1/V2 y resumir el resto mediante referencias; no borrar distinciones de entorno.</x:v>
+      </x:c>
       <x:c r="P23" s="10" t="str"/>
       <x:c r="Q23" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1876,18 +1958,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I24" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J24" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K24" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L24" s="10" t="str"/>
-      <x:c r="M24" s="10" t="str"/>
-      <x:c r="N24" s="10" t="str"/>
-      <x:c r="O24" s="10" t="str"/>
+        <x:v>Edición de validación profesional</x:v>
+      </x:c>
+      <x:c r="L24" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M24" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.11; appendices/anexo_h_validacion_profesional.tex §§H.3–H.6</x:v>
+      </x:c>
+      <x:c r="N24" s="10" t="str">
+        <x:v>Capítulo y Anexo H repiten tablas de sesiones, fichas y limitaciones; Anexo H debe ser el detalle y capítulo el resumen.</x:v>
+      </x:c>
+      <x:c r="O24" s="10" t="str">
+        <x:v>Conservar síntesis en resultados y dejar fichas/evidencia en Anexo H; revisar duplicaciones internas del anexo.</x:v>
+      </x:c>
       <x:c r="P24" s="10" t="str"/>
       <x:c r="Q24" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1925,18 +2015,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I25" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J25" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K25" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L25" s="10" t="str"/>
-      <x:c r="M25" s="10" t="str"/>
-      <x:c r="N25" s="10" t="str"/>
-      <x:c r="O25" s="10" t="str"/>
+        <x:v>Edición de requerimientos y límites</x:v>
+      </x:c>
+      <x:c r="L25" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M25" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex; chapters/capitulo_13_resultados_evaluacion.tex §13.12</x:v>
+      </x:c>
+      <x:c r="N25" s="10" t="str">
+        <x:v>La ausencia de comparación independiente y de validación clínica se expresa repetidamente; parte de esa reiteración protege contra interpretar métricas como evidencia clínica.</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="str">
+        <x:v>Definir una explicación canónica y evitar suprimir advertencias locales necesarias para interpretar cada resultado.</x:v>
+      </x:c>
       <x:c r="P25" s="10" t="str"/>
       <x:c r="Q25" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -1974,18 +2072,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I26" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J26" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K26" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L26" s="10" t="str"/>
-      <x:c r="M26" s="10" t="str"/>
-      <x:c r="N26" s="10" t="str"/>
-      <x:c r="O26" s="10" t="str"/>
+        <x:v>Edición de requerimientos</x:v>
+      </x:c>
+      <x:c r="L26" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M26" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex §§9.7, 9.10; chapters/capitulo_10_diseno_arquitectura.tex §§10.4.2–10.5</x:v>
+      </x:c>
+      <x:c r="N26" s="10" t="str">
+        <x:v>RF-15/RF-23 y RF-05/RF-25 presentan solapamiento; modelo Patient/subjectRef también se explica en varias secciones.</x:v>
+      </x:c>
+      <x:c r="O26" s="10" t="str">
+        <x:v>Consolidar requisitos solo tras comparar criterios de aceptación y conservar toda trazabilidad ID.</x:v>
+      </x:c>
       <x:c r="P26" s="10" t="str"/>
       <x:c r="Q26" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2023,18 +2129,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I27" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K27" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L27" s="10" t="str"/>
-      <x:c r="M27" s="10" t="str"/>
-      <x:c r="N27" s="10" t="str"/>
-      <x:c r="O27" s="10" t="str"/>
+        <x:v>Referencias cruzadas</x:v>
+      </x:c>
+      <x:c r="L27" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M27" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex §9.1; chapters/capitulo_10_diseno_arquitectura.tex §10.8; chapters/capitulo_11_capacidades_prototipo.tex §11.8; chapters/capitulo_14_planificacion_academica.tex; appendices/anexo_c_modulo_axial_preliminar.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N27" s="10" t="str">
+        <x:v>§10.8 remite a vista de procesos 10.4.1, mientras ese apartado está en 10.5; se detectan referencias cruzadas manuales adicionales en el listado del hallazgo.</x:v>
+      </x:c>
+      <x:c r="O27" s="10" t="str">
+        <x:v>Migrar remisiones a labels automáticos y comprobar los destinos en PDF.</x:v>
+      </x:c>
       <x:c r="P27" s="10" t="str"/>
       <x:c r="Q27" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2072,18 +2186,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I28" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J28" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K28" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L28" s="10" t="str"/>
-      <x:c r="M28" s="10" t="str"/>
-      <x:c r="N28" s="10" t="str"/>
-      <x:c r="O28" s="10" t="str"/>
+        <x:v>Trazabilidad de requisitos</x:v>
+      </x:c>
+      <x:c r="L28" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M28" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex §§9.2, 9.10</x:v>
+      </x:c>
+      <x:c r="N28" s="10" t="str">
+        <x:v>La regla “cada requerimiento nace de una necesidad” no describe bien requisitos derivados de seguridad/estado del arte; la matriz de trazabilidad debe cotejarse contra todas las filas del capítulo.</x:v>
+      </x:c>
+      <x:c r="O28" s="10" t="str">
+        <x:v>Identificar la fuente de cada requisito y completar trazabilidad, sin atribuir una necesidad de usuario inexistente.</x:v>
+      </x:c>
       <x:c r="P28" s="10" t="str"/>
       <x:c r="Q28" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2121,18 +2243,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I29" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K29" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L29" s="10" t="str"/>
-      <x:c r="M29" s="10" t="str"/>
-      <x:c r="N29" s="10" t="str"/>
-      <x:c r="O29" s="10" t="str"/>
+        <x:v>Estado de infraestructura</x:v>
+      </x:c>
+      <x:c r="L29" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M29" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §§10.3, 10.5.2, 10.6.3, 10.7.3; ADR-007</x:v>
+      </x:c>
+      <x:c r="N29" s="10" t="str">
+        <x:v>El capítulo mezcla arquitectura objetivo, planificada y despliegue/validación observados; el texto posterior identifica DEV V2 validado dentro de alcance base.</x:v>
+      </x:c>
+      <x:c r="O29" s="10" t="str">
+        <x:v>Usar estados temporales precisos: diseñado, desplegado, probado y no productivo; enlazar evidencia de cada componente.</x:v>
+      </x:c>
       <x:c r="P29" s="10" t="str"/>
       <x:c r="Q29" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2170,18 +2300,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K30" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L30" s="10" t="str"/>
-      <x:c r="M30" s="10" t="str"/>
-      <x:c r="N30" s="10" t="str"/>
-      <x:c r="O30" s="10" t="str"/>
+        <x:v>Atribución de evidencia</x:v>
+      </x:c>
+      <x:c r="L30" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M30" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §10.9.4; chapters/capitulo_08_user_research.tex tablas de encuesta/confianza; Anexo D</x:v>
+      </x:c>
+      <x:c r="N30" s="10" t="str">
+        <x:v>Coincide con H53: la atribución plural de rechazo de confianza numérica no refleja las opiniones divergentes; además la encuesta valora confianza/transparencia.</x:v>
+      </x:c>
+      <x:c r="O30" s="10" t="str">
+        <x:v>Resolver junto con H53 y distinguir puntaje calibrado de estado operativo.</x:v>
+      </x:c>
       <x:c r="P30" s="10" t="str"/>
       <x:c r="Q30" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2219,18 +2357,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I31" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K31" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L31" s="10" t="str"/>
-      <x:c r="M31" s="10" t="str"/>
-      <x:c r="N31" s="10" t="str"/>
-      <x:c r="O31" s="10" t="str"/>
+        <x:v>Metodología de validación</x:v>
+      </x:c>
+      <x:c r="L31" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M31" s="10" t="str">
+        <x:v>chapters/capitulo_05_alcance.tex §5.3; chapters/capitulo_08_user_research.tex; chapters/capitulo_12_metodologia_validacion.tex; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
+      </x:c>
+      <x:c r="N31" s="10" t="str">
+        <x:v>Se organizan en distintos pasajes bloques de alcance, niveles técnicos, capas de prueba y tipos de validación, sin una única taxonomía común.</x:v>
+      </x:c>
+      <x:c r="O31" s="10" t="str">
+        <x:v>Acordar un mapa de niveles con nombres y alcance explícitos y referenciarlo, distinguiéndolo de las capas de test.</x:v>
+      </x:c>
       <x:c r="P31" s="10" t="str"/>
       <x:c r="Q31" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2268,18 +2414,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K32" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L32" s="10" t="str"/>
-      <x:c r="M32" s="10" t="str"/>
-      <x:c r="N32" s="10" t="str"/>
-      <x:c r="O32" s="10" t="str"/>
+        <x:v>Encuesta y población</x:v>
+      </x:c>
+      <x:c r="L32" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M32" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex §§8.11.1–8.11.2; archivos fuente del cuestionario/datos por localizar</x:v>
+      </x:c>
+      <x:c r="N32" s="10" t="str">
+        <x:v>El texto informa 167 respuestas, pero en este repositorio no se localizó un cuestionario ni tabulación por ítem que permita reconstruir elegibilidad, exclusiones y denominadores.</x:v>
+      </x:c>
+      <x:c r="O32" s="10" t="str">
+        <x:v>Solicitar/localizar cuestionario y exportación agregada original; no reconstruir respuestas ni denominadores desde porcentajes del PDF.</x:v>
+      </x:c>
       <x:c r="P32" s="10" t="str"/>
       <x:c r="Q32" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2317,18 +2471,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K33" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L33" s="10" t="str"/>
-      <x:c r="M33" s="10" t="str"/>
-      <x:c r="N33" s="10" t="str"/>
-      <x:c r="O33" s="10" t="str"/>
+        <x:v>Estado de evaluación axial</x:v>
+      </x:c>
+      <x:c r="L33" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M33" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.10 y tabla de estado; chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.4</x:v>
+      </x:c>
+      <x:c r="N33" s="10" t="str">
+        <x:v>El resultado axial está debajo del gate y no se considera baseline; el fuente también describe co-registro nativo T1/T2, afirmación distinta de registro entre SPIDER y dataset axial.</x:v>
+      </x:c>
+      <x:c r="O33" s="10" t="str">
+        <x:v>Ajustar cualquier uso ambiguo de “validado” a “evaluado”; separar co-registro T1/T2 intra-dataset de registro multiplanar entre datasets.</x:v>
+      </x:c>
       <x:c r="P33" s="10" t="str"/>
       <x:c r="Q33" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2366,18 +2528,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I34" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K34" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L34" s="10" t="str"/>
-      <x:c r="M34" s="10" t="str"/>
-      <x:c r="N34" s="10" t="str"/>
-      <x:c r="O34" s="10" t="str"/>
+        <x:v>Terminología y estados</x:v>
+      </x:c>
+      <x:c r="L34" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M34" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex; chapters/capitulo_09_requerimientos.tex; chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_11_capacidades_prototipo.tex</x:v>
+      </x:c>
+      <x:c r="N34" s="10" t="str">
+        <x:v>Se usan denominaciones variables para el dataset axial, regiones anatómicas y estados de revisión; el glosario contiene entradas relacionadas, pero no unifica todos los contratos.</x:v>
+      </x:c>
+      <x:c r="O34" s="10" t="str">
+        <x:v>Definir términos preferidos y estados de revisión en glosario/contrato; armonizar el uso en prosa y tablas.</x:v>
+      </x:c>
       <x:c r="P34" s="10" t="str"/>
       <x:c r="Q34" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2415,18 +2585,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I35" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K35" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L35" s="10" t="str"/>
-      <x:c r="M35" s="10" t="str"/>
-      <x:c r="N35" s="10" t="str"/>
-      <x:c r="O35" s="10" t="str"/>
+        <x:v>Edición de documento final</x:v>
+      </x:c>
+      <x:c r="L35" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M35" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.2; chapters/capitulo_12_metodologia_validacion.tex §12.6; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N35" s="10" t="str">
+        <x:v>Se encuentran referencias a entregas previas, decisiones de proceso y frases de revisión editorial que no describen resultados actuales.</x:v>
+      </x:c>
+      <x:c r="O35" s="10" t="str">
+        <x:v>Mover la historia necesaria a anexos cronológicos y convertir el resto en descripción del estado actual.</x:v>
+      </x:c>
       <x:c r="P35" s="10" t="str"/>
       <x:c r="Q35" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2464,21 +2642,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I36" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L36" s="10" t="str"/>
-      <x:c r="M36" s="10" t="str"/>
-      <x:c r="N36" s="10" t="str"/>
-      <x:c r="O36" s="10" t="str"/>
-      <x:c r="P36" s="10" t="str"/>
+        <x:v>Referencias anatómicas y clínicas</x:v>
+      </x:c>
+      <x:c r="L36" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M36" s="10" t="str">
+        <x:v>chapters/capitulo_11_capacidades_prototipo.tex §11.5; chapters/capitulo_13_resultados_evaluacion.tex §13.6, Tabla 13.3; chapters/capitulo_07_marco_teorico.tex §7.8.2</x:v>
+      </x:c>
+      <x:c r="N36" s="10" t="str">
+        <x:v>Se retiró la comparación directa de suma angular L1–L5 con rango global de lordosis. Fuentes distinguen métodos/segmentos; el contenido actual no incluye la afirmación de altura discal 8–12 mm.</x:v>
+      </x:c>
+      <x:c r="O36" s="10" t="str">
+        <x:v>Usar mismos puntos anatómicos antes de cualquier comparación; no interpretar 36° como anormal.</x:v>
+      </x:c>
+      <x:c r="P36" s="10" t="str">
+        <x:v>1126134521c79d5858b220c5a163e0dd7f84610e</x:v>
+      </x:c>
       <x:c r="Q36" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R36" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -2513,18 +2701,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I37" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L37" s="10" t="str"/>
-      <x:c r="M37" s="10" t="str"/>
-      <x:c r="N37" s="10" t="str"/>
-      <x:c r="O37" s="10" t="str"/>
+        <x:v>Comparación de modelos</x:v>
+      </x:c>
+      <x:c r="L37" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M37" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.4.1; chapters/capitulo_07_marco_teorico.tex §7.7.4; chapters/capitulo_13_resultados_evaluacion.tex §13.3</x:v>
+      </x:c>
+      <x:c r="N37" s="10" t="str">
+        <x:v>SPINEPS/nnU-Net figuran como antecedentes o comparadores; el 0,893 informado proviene de la evaluación propia y no incluye comparación reproducida contra sus resultados.</x:v>
+      </x:c>
+      <x:c r="O37" s="10" t="str">
+        <x:v>Presentarlos como antecedentes, no benchmark comparativo, salvo que se adopte partición/protocolo realmente comparable.</x:v>
+      </x:c>
       <x:c r="P37" s="10" t="str"/>
       <x:c r="Q37" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2562,18 +2758,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I38" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L38" s="10" t="str"/>
-      <x:c r="M38" s="10" t="str"/>
-      <x:c r="N38" s="10" t="str"/>
-      <x:c r="O38" s="10" t="str"/>
+        <x:v>Ecuaciones y formato</x:v>
+      </x:c>
+      <x:c r="L38" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M38" s="10" t="str">
+        <x:v>chapters/capitulo_07_marco_teorico.tex §§7.9.2–7.9.4; chapters/capitulo_08_user_research.tex §8.11.1; chapters/capitulo_15_modelo_negocio.tex §§14.6, 14.8</x:v>
+      </x:c>
+      <x:c r="N38" s="10" t="str">
+        <x:v>Los números de ecuación se repiten por capítulo y hay símbolos/formatos reportados por el tutor que requieren inspección renderizada del PDF.</x:v>
+      </x:c>
+      <x:c r="O38" s="10" t="str">
+        <x:v>Numerar ecuaciones por capítulo y verificar símbolos y exponentes visualmente antes del PDF de cierre.</x:v>
+      </x:c>
       <x:c r="P38" s="10" t="str"/>
       <x:c r="Q38" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2611,18 +2815,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I39" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L39" s="10" t="str"/>
-      <x:c r="M39" s="10" t="str"/>
-      <x:c r="N39" s="10" t="str"/>
-      <x:c r="O39" s="10" t="str"/>
+        <x:v>Tablas e índices</x:v>
+      </x:c>
+      <x:c r="L39" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M39" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex; chapters/capitulo_09_requerimientos.tex; chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_11_capacidades_prototipo.tex; chapters/capitulo_13_resultados_evaluacion.tex; appendices/anexo_f_evolucion_tecnica.tex</x:v>
+      </x:c>
+      <x:c r="N39" s="10" t="str">
+        <x:v>El fuente incluye tablas con y sin caption y el índice se genera desde captions; se reproduce el problema de referencias manuales y formato heterogéneo descrito por el tutor.</x:v>
+      </x:c>
+      <x:c r="O39" s="10" t="str">
+        <x:v>Inventariar cada tabla, rotular y normalizar de forma consistente; reconstruir listas en compilación final.</x:v>
+      </x:c>
       <x:c r="P39" s="10" t="str"/>
       <x:c r="Q39" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2660,18 +2872,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I40" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L40" s="10" t="str"/>
-      <x:c r="M40" s="10" t="str"/>
-      <x:c r="N40" s="10" t="str"/>
-      <x:c r="O40" s="10" t="str"/>
+        <x:v>Índice y jerarquía</x:v>
+      </x:c>
+      <x:c r="L40" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M40" s="10" t="str">
+        <x:v>main.tex; chapters/capitulo_05_alcance.tex; chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_14_planificacion_academica.tex; appendices/anexo_c_modulo_axial_preliminar.tex; appendices/anexo_h_validacion_profesional.tex</x:v>
+      </x:c>
+      <x:c r="N40" s="10" t="str">
+        <x:v>La estructura se genera desde headings, pero hay remisiones y títulos que deben cotejarse contra PDF; el texto fuente contiene al menos secciones de proceso no aptas como contenido final.</x:v>
+      </x:c>
+      <x:c r="O40" s="10" t="str">
+        <x:v>Revisar niveles de headings, entradas de índice y títulos contra PDF recompilado, no editar números impresos manualmente.</x:v>
+      </x:c>
       <x:c r="P40" s="10" t="str"/>
       <x:c r="Q40" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2709,18 +2929,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I41" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L41" s="10" t="str"/>
-      <x:c r="M41" s="10" t="str"/>
-      <x:c r="N41" s="10" t="str"/>
-      <x:c r="O41" s="10" t="str"/>
+        <x:v>Corrección de estilo</x:v>
+      </x:c>
+      <x:c r="L41" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M41" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex §9.9; chapters/capitulo_11_capacidades_prototipo.tex; chapters/capitulo_14_planificacion_academica.tex</x:v>
+      </x:c>
+      <x:c r="N41" s="10" t="str">
+        <x:v>Se reproducen giros gramaticales internos (“no se dependen”) y estados en futuro condicional para capacidades descritas como implementadas.</x:v>
+      </x:c>
+      <x:c r="O41" s="10" t="str">
+        <x:v>Corregir idioma/tiempos verbales tras verificar cada estado contra evidencia del repositorio.</x:v>
+      </x:c>
       <x:c r="P41" s="10" t="str"/>
       <x:c r="Q41" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2758,18 +2986,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I42" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L42" s="10" t="str"/>
-      <x:c r="M42" s="10" t="str"/>
-      <x:c r="N42" s="10" t="str"/>
-      <x:c r="O42" s="10" t="str"/>
+        <x:v>Glosario e idioma técnico</x:v>
+      </x:c>
+      <x:c r="L42" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M42" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex; chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_13_resultados_evaluacion.tex; appendices/anexo_b_glosario.tex</x:v>
+      </x:c>
+      <x:c r="N42" s="10" t="str">
+        <x:v>Hay uso recurrente de anglicismos y códigos de implementación; las tablas mezclan estados en inglés con el cuerpo en español.</x:v>
+      </x:c>
+      <x:c r="O42" s="10" t="str">
+        <x:v>Definir siglas y términos en primera aparición/glosario; mantener códigos internos solo donde aporten trazabilidad.</x:v>
+      </x:c>
       <x:c r="P42" s="10" t="str"/>
       <x:c r="Q42" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2807,18 +3043,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I43" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L43" s="10" t="str"/>
-      <x:c r="M43" s="10" t="str"/>
-      <x:c r="N43" s="10" t="str"/>
-      <x:c r="O43" s="10" t="str"/>
+        <x:v>Estructura de anexos</x:v>
+      </x:c>
+      <x:c r="L43" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M43" s="10" t="str">
+        <x:v>appendices/anexo_a_glosario_tecnico.tex; appendices/anexo_b_glosario.tex; appendices/anexo_c_modulo_axial_preliminar.tex; appendices/anexo_f_evolucion_tecnica.tex; appendices/anexo_h_validacion_profesional.tex</x:v>
+      </x:c>
+      <x:c r="N43" s="10" t="str">
+        <x:v>Los anexos siguen convenciones distintas de encabezado; C agrupa dataset, origen y alcance; validar viñeta huérfana en el PDF renderizado.</x:v>
+      </x:c>
+      <x:c r="O43" s="10" t="str">
+        <x:v>Homogeneizar títulos/niveles y ordenar glosario; verificar la primera página del Anexo H en el PDF.</x:v>
+      </x:c>
       <x:c r="P43" s="10" t="str"/>
       <x:c r="Q43" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2856,18 +3100,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I44" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J44" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L44" s="10" t="str"/>
-      <x:c r="M44" s="10" t="str"/>
-      <x:c r="N44" s="10" t="str"/>
-      <x:c r="O44" s="10" t="str"/>
+        <x:v>Autoría y contribuciones</x:v>
+      </x:c>
+      <x:c r="L44" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M44" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §10.6.1; chapters/capitulo_12_metodologia_validacion.tex §12.1</x:v>
+      </x:c>
+      <x:c r="N44" s="10" t="str">
+        <x:v>Las referencias a “un integrante” y “el otro” no identifican autor ni explicitan aportes.</x:v>
+      </x:c>
+      <x:c r="O44" s="10" t="str">
+        <x:v>Agregar tabla de contribuciones solo con evidencia de autoría verificable; evitar inferir roles personales.</x:v>
+      </x:c>
       <x:c r="P44" s="10" t="str"/>
       <x:c r="Q44" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2905,18 +3157,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I45" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J45" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K45" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L45" s="10" t="str"/>
-      <x:c r="M45" s="10" t="str"/>
-      <x:c r="N45" s="10" t="str"/>
-      <x:c r="O45" s="10" t="str"/>
+        <x:v>Disponibilidad y sanitización</x:v>
+      </x:c>
+      <x:c r="L45" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M45" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §§10.7.1–10.7.2; chapters/capitulo_13_resultados_evaluacion.tex §13.9</x:v>
+      </x:c>
+      <x:c r="N45" s="10" t="str">
+        <x:v>Se imprimen identificadores de proyectos, revisión y detalles de costo/configuración; el valor de reproducibilidad debe preservarse sin publicar secretos o datos personales innecesarios.</x:v>
+      </x:c>
+      <x:c r="O45" s="10" t="str">
+        <x:v>Revisar qué identificadores son públicos/necesarios y trasladar hashes/licencias/instrucciones a una disponibilidad reproducible; nunca eliminar trazabilidad de evidencia.</x:v>
+      </x:c>
       <x:c r="P45" s="10" t="str"/>
       <x:c r="Q45" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -2954,18 +3214,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I46" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J46" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K46" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L46" s="10" t="str"/>
-      <x:c r="M46" s="10" t="str"/>
-      <x:c r="N46" s="10" t="str"/>
-      <x:c r="O46" s="10" t="str"/>
+        <x:v>Privacidad y ética de entrevistas</x:v>
+      </x:c>
+      <x:c r="L46" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M46" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex §8.3; appendices/anexo_d_entrevistas.tex D.1–D.5; documentos de consentimiento por localizar</x:v>
+      </x:c>
+      <x:c r="N46" s="10" t="str">
+        <x:v>Los anexos incluyen nombres, matrículas, referencias profesionales y transcripciones; el paquete no contiene consentimiento ni fechas fuente suficientes para autorizar nuevas afirmaciones o agradecimientos.</x:v>
+      </x:c>
+      <x:c r="O46" s="10" t="str">
+        <x:v>No publicar detalles personales adicionales ni completar consentimientos retroactivamente; localizar autorizaciones existentes y limitar la versión a evidencia autorizada.</x:v>
+      </x:c>
       <x:c r="P46" s="10" t="str"/>
       <x:c r="Q46" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3003,18 +3271,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I47" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J47" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K47" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L47" s="10" t="str"/>
-      <x:c r="M47" s="10" t="str"/>
-      <x:c r="N47" s="10" t="str"/>
-      <x:c r="O47" s="10" t="str"/>
+        <x:v>Evidencia de resultados</x:v>
+      </x:c>
+      <x:c r="L47" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M47" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.6; artifacts de evaluación por localizar</x:v>
+      </x:c>
+      <x:c r="N47" s="10" t="str">
+        <x:v>Los resultados no ofrecen figuras de comparación máscara/referencia ni dispersión por paciente; tampoco se identificó un artefacto con intervalos de confianza/bootstrap en el documento auditado.</x:v>
+      </x:c>
+      <x:c r="O47" s="10" t="str">
+        <x:v>Agregar solo visualizaciones y métricas reconstruibles desde predicciones/anotaciones verificables; no generar intervalos sin datos fuente.</x:v>
+      </x:c>
       <x:c r="P47" s="10" t="str"/>
       <x:c r="Q47" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3052,18 +3328,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J48" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K48" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L48" s="10" t="str"/>
-      <x:c r="M48" s="10" t="str"/>
-      <x:c r="N48" s="10" t="str"/>
-      <x:c r="O48" s="10" t="str"/>
+        <x:v>Requisitos no funcionales</x:v>
+      </x:c>
+      <x:c r="L48" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M48" s="10" t="str">
+        <x:v>chapters/capitulo_09_requerimientos.tex RNF-02 y RNF-10; chapters/capitulo_13_resultados_evaluacion.tex §13.9</x:v>
+      </x:c>
+      <x:c r="N48" s="10" t="str">
+        <x:v>RNF-02/RNF-10 no fijan umbrales cuantitativos reproducibles; la mediana citada en resultados no se presenta como criterio de aceptación.</x:v>
+      </x:c>
+      <x:c r="O48" s="10" t="str">
+        <x:v>Distinguir requisito medible de resultado observado; definir metas solo si la evidencia y el alcance las sostienen.</x:v>
+      </x:c>
       <x:c r="P48" s="10" t="str"/>
       <x:c r="Q48" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3101,18 +3385,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I49" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J49" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K49" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L49" s="10" t="str"/>
-      <x:c r="M49" s="10" t="str"/>
-      <x:c r="N49" s="10" t="str"/>
-      <x:c r="O49" s="10" t="str"/>
+        <x:v>Consistencia financiera</x:v>
+      </x:c>
+      <x:c r="L49" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M49" s="10" t="str">
+        <x:v>chapters/capitulo_15_modelo_negocio.tex §§14.5, 14.11–14.12; financial/</x:v>
+      </x:c>
+      <x:c r="N49" s="10" t="str">
+        <x:v>La memoria apunta diferencias entre perturbaciones declaradas y aumentos observados, magnitud de costos y unidades; deben recalcularse con el libro canónico antes de ajustar textos.</x:v>
+      </x:c>
+      <x:c r="O49" s="10" t="str">
+        <x:v>Reconciliar fórmulas y escenarios con workbook canónico, comentar valores extremos y normalizar formato numérico.</x:v>
+      </x:c>
       <x:c r="P49" s="10" t="str"/>
       <x:c r="Q49" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3150,18 +3442,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I50" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J50" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K50" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L50" s="10" t="str"/>
-      <x:c r="M50" s="10" t="str"/>
-      <x:c r="N50" s="10" t="str"/>
-      <x:c r="O50" s="10" t="str"/>
+        <x:v>Riesgos de negocio</x:v>
+      </x:c>
+      <x:c r="L50" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M50" s="10" t="str">
+        <x:v>chapters/capitulo_15_modelo_negocio.tex §15.4</x:v>
+      </x:c>
+      <x:c r="N50" s="10" t="str">
+        <x:v>La sección enumera riesgos sin probabilidad, impacto ni mitigaciones comparables.</x:v>
+      </x:c>
+      <x:c r="O50" s="10" t="str">
+        <x:v>Crear matriz cualitativa probabilidad-impacto-mitigación con supuestos declarados, sin asignar probabilidades cuantitativas inventadas.</x:v>
+      </x:c>
       <x:c r="P50" s="10" t="str"/>
       <x:c r="Q50" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3199,18 +3499,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I51" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J51" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K51" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L51" s="10" t="str"/>
-      <x:c r="M51" s="10" t="str"/>
-      <x:c r="N51" s="10" t="str"/>
-      <x:c r="O51" s="10" t="str"/>
+        <x:v>Bibliografía y glosario</x:v>
+      </x:c>
+      <x:c r="L51" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M51" s="10" t="str">
+        <x:v>appendices/anexo_b_glosario.tex; references.bib; chapters/capitulo_06_estado_del_arte.tex §§6.5–6.8; chapters/capitulo_15_modelo_negocio.tex §14.7</x:v>
+      </x:c>
+      <x:c r="N51" s="10" t="str">
+        <x:v>Hay siglas técnicas usadas sin glosario y herramientas/costos con referencias incompletas; DOI y metadatos de varias citas aún requieren contraste primario.</x:v>
+      </x:c>
+      <x:c r="O51" s="10" t="str">
+        <x:v>Verificar referencias una a una en sus fuentes/editoriales; no añadir citas sin confirmar pertinencia y metadatos.</x:v>
+      </x:c>
       <x:c r="P51" s="10" t="str"/>
       <x:c r="Q51" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3248,18 +3556,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I52" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J52" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K52" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L52" s="10" t="str"/>
-      <x:c r="M52" s="10" t="str"/>
-      <x:c r="N52" s="10" t="str"/>
-      <x:c r="O52" s="10" t="str"/>
+        <x:v>Presentación de marca</x:v>
+      </x:c>
+      <x:c r="L52" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M52" s="10" t="str">
+        <x:v>chapters/capitulo_14_planificacion_academica.tex §14.2.1</x:v>
+      </x:c>
+      <x:c r="N52" s="10" t="str">
+        <x:v>La explicación de marca y sistema visual es extensa y el nombre aparece en el tramo financiero sin presentación temprana.</x:v>
+      </x:c>
+      <x:c r="O52" s="10" t="str">
+        <x:v>Reducir o mover el detalle de branding y presentar el nombre en introducción/alcance si se conserva.</x:v>
+      </x:c>
       <x:c r="P52" s="10" t="str"/>
       <x:c r="Q52" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3297,18 +3613,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I53" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J53" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K53" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L53" s="10" t="str"/>
-      <x:c r="M53" s="10" t="str"/>
-      <x:c r="N53" s="10" t="str"/>
-      <x:c r="O53" s="10" t="str"/>
+        <x:v>Pulido editorial de estado del arte</x:v>
+      </x:c>
+      <x:c r="L53" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M53" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.10; tablas 6.3–6.4</x:v>
+      </x:c>
+      <x:c r="N53" s="10" t="str">
+        <x:v>El apartado sobre imagen axial repite el plano en la enumeración; hay errores terminológicos menores y una caracterización vaga de la propuesta Perumal.</x:v>
+      </x:c>
+      <x:c r="O53" s="10" t="str">
+        <x:v>Corregir duplicación y precisión terminológica; atribuir la propuesta técnica con fuente y alcance concretos.</x:v>
+      </x:c>
       <x:c r="P53" s="10" t="str"/>
       <x:c r="Q53" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3346,21 +3670,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I54" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J54" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K54" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L54" s="10" t="str"/>
-      <x:c r="M54" s="10" t="str"/>
-      <x:c r="N54" s="10" t="str"/>
-      <x:c r="O54" s="10" t="str"/>
-      <x:c r="P54" s="10" t="str"/>
+        <x:v>Atribución de evidencia</x:v>
+      </x:c>
+      <x:c r="L54" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M54" s="10" t="str">
+        <x:v>chapters/capitulo_10_diseno_arquitectura.tex §10.9.4; appendices/anexo_d_entrevistas.tex §§D.1–D.3</x:v>
+      </x:c>
+      <x:c r="N54" s="10" t="str">
+        <x:v>La frase vigente atribuye a “las entrevistas” que mostrar confianza numérica induce interpretación indebida. En D.1 EN-01 advierte sesgo al recibir una graduación IA; EN-02/D.2 y EN-03/D.3 consideran útil mostrar confianza.</x:v>
+      </x:c>
+      <x:c r="O54" s="10" t="str">
+        <x:v>Corregir atribución plural; distinguir la preocupación de EN-01 de las opiniones favorables y presentar la decisión como criterio de diseño con fundamento metodológico.</x:v>
+      </x:c>
+      <x:c r="P54" s="10" t="str">
+        <x:v>44a2481734bfe47d3d344fe8479af1b33ac198a7</x:v>
+      </x:c>
       <x:c r="Q54" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R54" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3395,21 +3729,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I55" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J55" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K55" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L55" s="10" t="str"/>
-      <x:c r="M55" s="10" t="str"/>
-      <x:c r="N55" s="10" t="str"/>
-      <x:c r="O55" s="10" t="str"/>
-      <x:c r="P55" s="10" t="str"/>
+        <x:v>Trazabilidad de cita</x:v>
+      </x:c>
+      <x:c r="L55" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M55" s="10" t="str">
+        <x:v>chapters/capitulo_07_marco_teorico.tex §7.10.2; chapters/capitulo_08_marco_teorico.tex; appendices/anexo_d_entrevistas.tex D.1–D.5</x:v>
+      </x:c>
+      <x:c r="N55" s="10" t="str">
+        <x:v>La frase “si se ve bonito no es lo que realmente importa” aparece en dos capítulos activos; no aparece en las cinco transcripciones D.1–D.5.</x:v>
+      </x:c>
+      <x:c r="O55" s="10" t="str">
+        <x:v>Retirar la cita textual o identificar una fuente primaria fechada y autorizada; conservar transcripciones sin cambios.</x:v>
+      </x:c>
+      <x:c r="P55" s="10" t="str">
+        <x:v>44a2481734bfe47d3d344fe8479af1b33ac198a7</x:v>
+      </x:c>
       <x:c r="Q55" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R55" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3444,21 +3788,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I56" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J56" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K56" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L56" s="10" t="str"/>
-      <x:c r="M56" s="10" t="str"/>
-      <x:c r="N56" s="10" t="str"/>
-      <x:c r="O56" s="10" t="str"/>
-      <x:c r="P56" s="10" t="str"/>
+        <x:v>User research / validación</x:v>
+      </x:c>
+      <x:c r="L56" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M56" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex Tabla 8.5 y §§8.5–8.6; chapters/capitulo_13_resultados_evaluacion.tex §§13.1, 13.12; chapters/capitulo_16_conclusiones.tex; appendices/anexo_d_entrevistas.tex D.5</x:v>
+      </x:c>
+      <x:c r="N56" s="10" t="str">
+        <x:v>EN-05 recomienda explícitamente comparar mediciones del sistema con mediciones de especialistas. La conclusión general ahora identifica la recomendación y registra que esa comparación no se ejecutó; la validación clínica/diagnóstica sigue fuera de la evidencia disponible.</x:v>
+      </x:c>
+      <x:c r="O56" s="10" t="str">
+        <x:v>La comparación independiente requerirá estudios comunes, especialistas y protocolo; no se presenta como realizada.</x:v>
+      </x:c>
+      <x:c r="P56" s="10" t="str">
+        <x:v>784066e6723fab9cb90bf5794783c3e667a1b415</x:v>
+      </x:c>
       <x:c r="Q56" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R56" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3493,18 +3847,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I57" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J57" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K57" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L57" s="10" t="str"/>
-      <x:c r="M57" s="10" t="str"/>
-      <x:c r="N57" s="10" t="str"/>
-      <x:c r="O57" s="10" t="str"/>
+        <x:v>Licencias y uso previsto</x:v>
+      </x:c>
+      <x:c r="L57" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M57" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.2; chapters/capitulo_11_capacidades_prototipo.tex §11.11.2; chapters/capitulo_15_modelo_negocio.tex; artifacts/manifests del clasificador subarticular</x:v>
+      </x:c>
+      <x:c r="N57" s="10" t="str">
+        <x:v>La tesis asocia LumbarDISC/RSNA a un clasificador y proyecta SaaS, pero falta análisis de términos del acuerdo aplicable, cadena de acceso/derivados y relación entre uso académico actual y uso comercial futuro. No se concluye incompatibilidad jurídica con la evidencia disponible.</x:v>
+      </x:c>
+      <x:c r="O57" s="10" t="str">
+        <x:v>Mantener bloqueado hasta adjuntar y revisar términos/licencias vigentes por dataset/modelo, alcance de redistribución y uso comercial; documentar límite sin emitir conclusión legal no sustentada.</x:v>
+      </x:c>
       <x:c r="P57" s="10" t="str"/>
       <x:c r="Q57" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3542,18 +3904,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I58" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J58" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K58" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L58" s="10" t="str"/>
-      <x:c r="M58" s="10" t="str"/>
-      <x:c r="N58" s="10" t="str"/>
-      <x:c r="O58" s="10" t="str"/>
+        <x:v>Comparabilidad de evaluación</x:v>
+      </x:c>
+      <x:c r="L58" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M58" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.1; chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.3; manifest sagital</x:v>
+      </x:c>
+      <x:c r="N58" s="10" t="str">
+        <x:v>La evaluación propia usa una partición 152/33/33; el benchmark SPIDER publica train/validation y un test oculto separado a nivel de paciente, con resultados de referencia. El 0,893 no es directamente comparable.</x:v>
+      </x:c>
+      <x:c r="O58" s="10" t="str">
+        <x:v>Reportar la partición como evaluación propia y reformular cualquier equivalencia con benchmark; no reentrenar ni acceder a test oculto sin protocolo.</x:v>
+      </x:c>
       <x:c r="P58" s="10" t="str"/>
       <x:c r="Q58" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3591,18 +3961,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I59" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J59" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K59" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L59" s="10" t="str"/>
-      <x:c r="M59" s="10" t="str"/>
-      <x:c r="N59" s="10" t="str"/>
-      <x:c r="O59" s="10" t="str"/>
+        <x:v>Estado del arte de clasificación</x:v>
+      </x:c>
+      <x:c r="L59" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M59" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.4.3; chapters/capitulo_11_capacidades_prototipo.tex §11.11.1; references.bib [6], [7]</x:v>
+      </x:c>
+      <x:c r="N59" s="10" t="str">
+        <x:v>SpineNet/SpineNetV2 cubren varias gradaciones degenerativas que se solapan con etiquetas discutidas; sin embargo, tareas, datos, licencias y condiciones de validación difieren del modelo PFI.</x:v>
+      </x:c>
+      <x:c r="O59" s="10" t="str">
+        <x:v>Actualizar el análisis como antecedente comparable y justificar por qué no se usa como baseline directo; no presentar sus métricas como comparación propia.</x:v>
+      </x:c>
       <x:c r="P59" s="10" t="str"/>
       <x:c r="Q59" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3640,21 +4018,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I60" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J60" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K60" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L60" s="10" t="str"/>
-      <x:c r="M60" s="10" t="str"/>
-      <x:c r="N60" s="10" t="str"/>
-      <x:c r="O60" s="10" t="str"/>
-      <x:c r="P60" s="10" t="str"/>
+        <x:v>Alineación bibliográfica clínica</x:v>
+      </x:c>
+      <x:c r="L60" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M60" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.4.4; chapters/capitulo_07_marco_teorico.tex §7.8.2; references.bib steurer_lumbar_stenosis_2011</x:v>
+      </x:c>
+      <x:c r="N60" s="10" t="str">
+        <x:v>La revisión de Steurer informa criterios AP/área variables y falta de consenso; ya no se afirma que el área sea más sensible.</x:v>
+      </x:c>
+      <x:c r="O60" s="10" t="str">
+        <x:v>Citar la revisión para describir criterios usados, no para inferir superioridad diagnóstica.</x:v>
+      </x:c>
+      <x:c r="P60" s="10" t="str">
+        <x:v>1126134521c79d5858b220c5a163e0dd7f84610e</x:v>
+      </x:c>
       <x:c r="Q60" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R60" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3689,21 +4077,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I61" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J61" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K61" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L61" s="10" t="str"/>
-      <x:c r="M61" s="10" t="str"/>
-      <x:c r="N61" s="10" t="str"/>
-      <x:c r="O61" s="10" t="str"/>
-      <x:c r="P61" s="10" t="str"/>
+        <x:v>Interpretación de medición</x:v>
+      </x:c>
+      <x:c r="L61" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M61" s="10" t="str">
+        <x:v>chapters/capitulo_13_resultados_evaluacion.tex §13.6, Tabla 13.3</x:v>
+      </x:c>
+      <x:c r="N61" s="10" t="str">
+        <x:v>El valor de 9,8 mm en L3–L4 se presenta como menor que uno de varios umbrales publicados (&lt;10 mm), expresamente no diagnóstico y sujeto a interpretación profesional.</x:v>
+      </x:c>
+      <x:c r="O61" s="10" t="str">
+        <x:v>No clasificar el estudio ni el método a partir de un único corte/medición.</x:v>
+      </x:c>
+      <x:c r="P61" s="10" t="str">
+        <x:v>1126134521c79d5858b220c5a163e0dd7f84610e</x:v>
+      </x:c>
       <x:c r="Q61" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R61" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3738,21 +4136,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I62" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J62" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K62" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L62" s="10" t="str"/>
-      <x:c r="M62" s="10" t="str"/>
-      <x:c r="N62" s="10" t="str"/>
-      <x:c r="O62" s="10" t="str"/>
-      <x:c r="P62" s="10" t="str"/>
+        <x:v>Panorama regulatorio comercial</x:v>
+      </x:c>
+      <x:c r="L62" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M62" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.7 y Tablas 6.2/6.6; references.bib</x:v>
+      </x:c>
+      <x:c r="N62" s="10" t="str">
+        <x:v>Se incorporaron decisiones FDA verificadas: CoLumbo K241211 (15-08-2024), MSKai K240793 (16-12-2024) y ScanDiags Ortho L-Spine MR-Q K242607 (21-02-2025). Los registros no se presentan como evidencia de equivalencia de indicación o desempeño con el PFI.</x:v>
+      </x:c>
+      <x:c r="O62" s="10" t="str">
+        <x:v>El inventario comercial completo y comparación de estudios clínicos siguen parciales; revisar cada resumen/indicación antes de comparaciones de desempeño.</x:v>
+      </x:c>
+      <x:c r="P62" s="10" t="str">
+        <x:v>475570dabc211261c0b8f6733bb197b910fb1b68</x:v>
+      </x:c>
       <x:c r="Q62" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R62" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3787,21 +4195,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I63" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J63" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K63" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L63" s="10" t="str"/>
-      <x:c r="M63" s="10" t="str"/>
-      <x:c r="N63" s="10" t="str"/>
-      <x:c r="O63" s="10" t="str"/>
-      <x:c r="P63" s="10" t="str"/>
+        <x:v>Metadatos bibliográficos y metodología</x:v>
+      </x:c>
+      <x:c r="L63" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M63" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.5 y Tabla 6.6; references.bib perumal_thecal_sac_2026</x:v>
+      </x:c>
+      <x:c r="N63" s="10" t="str">
+        <x:v>DOI y registro de PubMed/BMC: primer autor Akash Nixon; Perumal es último. La cita narrativa se corrigió y el antecedente ahora describe validación frente al promedio de dos radiólogos y MAE global 0,994 mm, sin trasladar sus resultados al PFI.</x:v>
+      </x:c>
+      <x:c r="O63" s="10" t="str">
+        <x:v>Usar el artículo como ejemplo metodológico externo, no como resultado propio ni umbral de aceptación del PFI.</x:v>
+      </x:c>
+      <x:c r="P63" s="10" t="str">
+        <x:v>475570dabc211261c0b8f6733bb197b910fb1b68</x:v>
+      </x:c>
       <x:c r="Q63" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R63" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3836,18 +4254,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I64" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J64" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K64" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L64" s="10" t="str"/>
-      <x:c r="M64" s="10" t="str"/>
-      <x:c r="N64" s="10" t="str"/>
-      <x:c r="O64" s="10" t="str"/>
+        <x:v>Procedencia de anotaciones axiales</x:v>
+      </x:c>
+      <x:c r="L64" s="10" t="str">
+        <x:v>Gestionador LaTeX; AI Module</x:v>
+      </x:c>
+      <x:c r="M64" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.3; chapters/capitulo_13_resultados_evaluacion.tex Tabla 13.1; manifests/notebooks axiales</x:v>
+      </x:c>
+      <x:c r="N64" s="10" t="str">
+        <x:v>515 pacientes y 1.545 máscaras se infieren como 3 niveles por paciente, pero el conteo observado y el universo de evaluación no están reconciliados con 81/102 casos; el paquete no contiene manifest concluyente.</x:v>
+      </x:c>
+      <x:c r="O64" s="10" t="str">
+        <x:v>Localizar release exacto, manifest y cuaderno; verificar máscaras y pacientes únicos antes de corregir conteos. No reconstruir cifras por multiplicación sola.</x:v>
+      </x:c>
       <x:c r="P64" s="10" t="str"/>
       <x:c r="Q64" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -3885,21 +4311,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I65" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J65" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="K65" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L65" s="10" t="str"/>
-      <x:c r="M65" s="10" t="str"/>
-      <x:c r="N65" s="10" t="str"/>
-      <x:c r="O65" s="10" t="str"/>
-      <x:c r="P65" s="10" t="str"/>
+        <x:v>Análisis de sustitutos y PACS</x:v>
+      </x:c>
+      <x:c r="L65" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M65" s="10" t="str">
+        <x:v>chapters/capitulo_06_estado_del_arte.tex §§6.6–6.8, Tablas 6.2/6.6; chapters/capitulo_08_user_research.tex Tabla 8.5; appendices/anexo_d_entrevistas.tex D.3, D.5</x:v>
+      </x:c>
+      <x:c r="N65" s="10" t="str">
+        <x:v>Las entrevistas EN-03/EN-05 describen delimitación de niveles y mediciones disponibles en sus PACS. Se añadió PACS nativo como sustituto parcial y se acotó el diferencial a integración, trazabilidad y revisión, sin afirmar superioridad comparativa.</x:v>
+      </x:c>
+      <x:c r="O65" s="10" t="str">
+        <x:v>Comparación directa de utilidad/esfuerzo contra los PACS de los centros no fue realizada.</x:v>
+      </x:c>
+      <x:c r="P65" s="10" t="str">
+        <x:v>475570dabc211261c0b8f6733bb197b910fb1b68</x:v>
+      </x:c>
       <x:c r="Q65" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R65" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3934,21 +4370,31 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I66" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J66" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K66" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L66" s="10" t="str"/>
-      <x:c r="M66" s="10" t="str"/>
-      <x:c r="N66" s="10" t="str"/>
-      <x:c r="O66" s="10" t="str"/>
-      <x:c r="P66" s="10" t="str"/>
+        <x:v>Alcance y preinforme</x:v>
+      </x:c>
+      <x:c r="L66" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M66" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex Tabla 8.5; chapters/capitulo_07_marco_teorico.tex §7.11.3; appendices/anexo_d_entrevistas.tex D.2, D.5</x:v>
+      </x:c>
+      <x:c r="N66" s="10" t="str">
+        <x:v>Se registraron las solicitudes de EN-02 sobre diferenciales y EN-05 sobre interpretación por nivel en lenguaje de informe; la decisión distingue esas demandas del preinforme geométrico editable y no diagnóstico actual.</x:v>
+      </x:c>
+      <x:c r="O66" s="10" t="str">
+        <x:v>No se implementa ni valida interpretación diagnóstica automática; decisión de alcance explícita.</x:v>
+      </x:c>
+      <x:c r="P66" s="10" t="str">
+        <x:v>784066e6723fab9cb90bf5794783c3e667a1b415</x:v>
+      </x:c>
       <x:c r="Q66" s="10" t="str">
-        <x:v>No evaluado</x:v>
+        <x:v>PDF recompilado: pdfLaTeX exit 0, 231 páginas; Biber 2.21 exit 0 en compilación limpia; sin referencias ni citas indefinidas. Revisión visual de tabla financiera (PDF p. 155).</x:v>
       </x:c>
       <x:c r="R66" s="10" t="str">
         <x:v>No revisado</x:v>
@@ -3983,18 +4429,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I67" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>Bloqueado por evidencia</x:v>
       </x:c>
       <x:c r="J67" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K67" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L67" s="10" t="str"/>
-      <x:c r="M67" s="10" t="str"/>
-      <x:c r="N67" s="10" t="str"/>
-      <x:c r="O67" s="10" t="str"/>
+        <x:v>Entrevistas, datos personales y método</x:v>
+      </x:c>
+      <x:c r="L67" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M67" s="10" t="str">
+        <x:v>chapters/capitulo_08_user_research.tex §§8.3–8.4; appendices/anexo_d_entrevistas.tex D.1–D.5</x:v>
+      </x:c>
+      <x:c r="N67" s="10" t="str">
+        <x:v>Las transcripciones no contienen fechas/duraciones para todas las sesiones; el texto aporta referencias de perfil cuyo soporte no está adjunto. No se puede confirmar consentimiento ni reconstruir metadata.</x:v>
+      </x:c>
+      <x:c r="O67" s="10" t="str">
+        <x:v>Limitar perfiles a datos respaldados por las fuentes disponibles; localizar fechas/consentimientos/autorización antes de publicar información personal adicional.</x:v>
+      </x:c>
       <x:c r="P67" s="10" t="str"/>
       <x:c r="Q67" s="10" t="str">
         <x:v>No evaluado</x:v>
@@ -4032,18 +4486,26 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I68" s="10" t="str">
-        <x:v>Sin revisar</x:v>
+        <x:v>En investigación</x:v>
       </x:c>
       <x:c r="J68" s="10" t="str">
-        <x:v>Por comprobar</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K68" s="10" t="str">
-        <x:v>Por clasificar</x:v>
-      </x:c>
-      <x:c r="L68" s="10" t="str"/>
-      <x:c r="M68" s="10" t="str"/>
-      <x:c r="N68" s="10" t="str"/>
-      <x:c r="O68" s="10" t="str"/>
+        <x:v>Verificación bibliográfica</x:v>
+      </x:c>
+      <x:c r="L68" s="10" t="str">
+        <x:v>Gestionador LaTeX</x:v>
+      </x:c>
+      <x:c r="M68" s="10" t="str">
+        <x:v>references.bib; referencias del capítulo 6 y marco teórico</x:v>
+      </x:c>
+      <x:c r="N68" s="10" t="str">
+        <x:v>No se ha completado la verificación primaria del conjunto [1]–[40]; la discrepancia de autoría en [9] ya está reproducida, pero el resto exige revisión DOI/título/volumen y soporte de afirmaciones.</x:v>
+      </x:c>
+      <x:c r="O68" s="10" t="str">
+        <x:v>Auditar todos los registros y sus afirmaciones enlazadas; corregir metadatos solo tras cotejo editorial/DOI.</x:v>
+      </x:c>
       <x:c r="P68" s="10" t="str"/>
       <x:c r="Q68" s="10" t="str">
         <x:v>No evaluado</x:v>

</xml_diff>

<commit_message>
audit(pfi): update evidence matrix and final PDF
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="Rfccff9b7e80c4f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rfb497684af094cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="R624eb0ce88804e70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" r:id="Rd93824da15784c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="2" r:id="Rf3aeac8541bf4462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="R63660d9db42c4a32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -447,7 +447,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"En investigación")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
         <x:v>No modificar Google Docs del tutor antes de la revisión final autorizada.</x:v>
@@ -475,7 +475,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIF(Seguimiento!I2:I68,"Corrección aplicada")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
         <x:v>No cerrar si faltan evidencias técnicas o pruebas exigidas.</x:v>
@@ -809,10 +809,10 @@
         <x:v>chapters/capitulo_10_diseno_arquitectura.tex; chapters/capitulo_12_metodologia_validacion.tex; main.pdf</x:v>
       </x:c>
       <x:c r="N4" s="10" t="str">
-        <x:v>Las cuatro figuras tienen archivos y captions activos; aparecen en la lista de figuras y en main.pdf (PDF pp. 88, 90, 99, 125). Se revisó visualmente cada página: no hay marcadores de inserción.</x:v>
+        <x:v>Las cuatro figuras están activas y legibles en el PDF recompilado; páginas físicas 94/96/105/132.</x:v>
       </x:c>
       <x:c r="O4" s="10" t="str">
-        <x:v>Cerrado con evidencia: las cuatro figuras cuestionadas aparecen en el PDF final con diagramas/captions activos y se revisaron visualmente las páginas físicas 93, 95, 104 y 131.</x:v>
+        <x:v>Sin cambios para H03; se conserva el baseline y se actualiza evidencia de QA.</x:v>
       </x:c>
       <x:c r="P4" s="10" t="str">
         <x:v>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</x:v>
@@ -870,10 +870,10 @@
         <x:v>chapters/capitulo_11_capacidades_prototipo.tex §11.4; chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.4; appendices/anexo_e_configuracion_entrenamiento.tex</x:v>
       </x:c>
       <x:c r="N5" s="10" t="str">
-        <x:v>La versión actual identifica seis clases, dos fondos, raw_0 y el gate axial oficial (Dice 0,679348; IoU 0,569973), y distingue la lectura secundaria (Dice 0,810566; IoU 0,691541). La tabla de resultados no publica los seis Dice por clase.</x:v>
+        <x:v>H04: el model card sagital publica solo Dice macro no-background 0.8934 e IoU macro 0.8080; no expone los tres Dice por clase. El model card axial sí trae métricas Dice/IoU por clase (raw_0 test Dice 0.1545; raw_50 0.9316; raw_100 0.8400; raw_150 0.7955; raw_200 0.6752). Gate axial no aprobado (macro foreground 0.67935). Evidencia: modelos/final/*.modelcard.md y *.manifest.json del snapshot AI.</x:v>
       </x:c>
       <x:c r="O5" s="10" t="str">
-        <x:v>Mantener el gate oficial y completar la tabla por clase con métricas provenientes del artifact verificable; no reinterpretar el promedio secundario como aprobado.</x:v>
+        <x:v>Completar solo las celdas de métrica que correspondan a cada modelo y dejar explícita la ausencia de desglose por clase para el modelo sagital. No volver a presentar el macro promedio como gate aprobado.</x:v>
       </x:c>
       <x:c r="P5" s="10" t="str"/>
       <x:c r="Q5" s="10" t="str">
@@ -1148,7 +1148,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="I10" s="10" t="str">
-        <x:v>En investigación</x:v>
+        <x:v>Corrección aplicada</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
         <x:v>Parcial</x:v>
@@ -1163,19 +1163,23 @@
         <x:v>chapters/capitulo_05_alcance.tex §5.5; chapters/capitulo_09_requerimientos.tex RF-08/RF-14; chapters/capitulo_11_capacidades_prototipo.tex §§11.1, 11.9; chapters/capitulo_13_resultados_evaluacion.tex</x:v>
       </x:c>
       <x:c r="N10" s="10" t="str">
-        <x:v>La fuente distingue Patient/patientId como dominio persistido en Backend y subjectRef como compatibilidad usada por historial/longitudinal en Frontend Demo. Debe verificarse el contrato y el comportamiento en snapshots para saber si RF-08 describe estado o intención.</x:v>
+        <x:v>Se cotejó el uso en snapshots: Patient/patientId para API y persistencia Backend; subjectRef continúa en historial/comparación del Frontend; Demo Mode es descriptivo, la gestión completa desde navegador sigue parcial. Se revisó y recompiló el texto en H09.</x:v>
       </x:c>
       <x:c r="O10" s="10" t="str">
-        <x:v>Mantener explícita la separación API/Frontend y ajustar estados de requisito a la evidencia de integración.</x:v>
-      </x:c>
-      <x:c r="P10" s="10" t="str"/>
+        <x:v>Reconciliar capítulos 3, 5, 8 y 9; no hubo cambio de código.</x:v>
+      </x:c>
+      <x:c r="P10" s="10" t="str">
+        <x:v>11568e2e8d5a80b6551288fbca74c6d13bb0ffa3</x:v>
+      </x:c>
       <x:c r="Q10" s="10" t="str">
-        <x:v>Revisión de código de los tres repositorios pendiente.</x:v>
+        <x:v>Compilación final: 232 páginas; sin undefined/fatal; revisión visual p.25. PDF SHA-256 A725AA2916F3739B1680E70EA5735A6D093B566BCDB8A6509D6B96A1F74251BB.</x:v>
       </x:c>
       <x:c r="R10" s="10" t="str">
         <x:v>No revisado</x:v>
       </x:c>
-      <x:c r="S10" s="10" t="str"/>
+      <x:c r="S10" s="10" t="str">
+        <x:v>Pendiente revisión final</x:v>
+      </x:c>
       <x:c r="T10" s="10" t="str"/>
       <x:c r="U10" s="10" t="str"/>
     </x:row>
@@ -1324,7 +1328,7 @@
         <x:v>Confirmado</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>Sí</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="K13" s="10" t="str">
         <x:v>Métricas y criterio de promoción</x:v>
@@ -1336,10 +1340,10 @@
         <x:v>chapters/capitulo_13_resultados_evaluacion.tex §§13.2–13.4; chapters/capitulo_07_marco_teorico.tex §7.9</x:v>
       </x:c>
       <x:c r="N13" s="10" t="str">
-        <x:v>El protocolo vigente exige IoU como condición; tabla de resultados informa IoU axial pero no para SPIDER sagital. HD95/NSD se explican teóricamente y no se reportan resultados.</x:v>
+        <x:v>H12: manifiestos/model cards contienen IoU agregada axial (test 0.56997 foreground; 0.69154 excluyendo raw_0) y sagital (0.8080 macro no-background). No se encontró HD95/NSD reportado en manifiestos ni model cards.</x:v>
       </x:c>
       <x:c r="O13" s="10" t="str">
-        <x:v>Recuperar IoU por modelo y reportarlo; si HD95 no existe, declararlo no calculado y revisar que el objetivo/criterio no prometa esa evidencia.</x:v>
+        <x:v>Mantener IoU vinculada a modelo, split y agregación. Declarar HD95/NSD no calculados; no inventar valores.</x:v>
       </x:c>
       <x:c r="P13" s="10" t="str"/>
       <x:c r="Q13" s="10" t="str">
@@ -1452,10 +1456,10 @@
         <x:v>chapters/capitulo_08_user_research.tex; chapters/capitulo_13_resultados_evaluacion.tex §13.11; appendices/anexo_d_entrevistas.tex; appendices/anexo_h_validacion_profesional.tex</x:v>
       </x:c>
       <x:c r="N15" s="10" t="str">
-        <x:v>Las descripciones de sesiones carecen de fechas verificables y el expediente disponible no acredita consentimientos ni autorizaciones para publicación. Se limita la redacción a las fuentes disponibles; no se recrearon metadatos.</x:v>
+        <x:v>H14: Anexo D contiene transcripciones documentales de entrevistas; no equivale a audios originales ni acredita fecha, consentimiento o autorización de uso/publicación.</x:v>
       </x:c>
       <x:c r="O15" s="10" t="str">
-        <x:v>Bloqueado hasta localizar registros fechados de sesiones, consentimientos y autorizaciones; no se inventaron metadatos ni se contactó a los profesionales.</x:v>
+        <x:v>Solicitar archivos originales de audio por sesión, registro fechado de cada sesión, consentimientos y autorizaciones de uso/publicación que correspondan.</x:v>
       </x:c>
       <x:c r="P15" s="10" t="str"/>
       <x:c r="Q15" s="10" t="str">
@@ -2429,10 +2433,10 @@
         <x:v>chapters/capitulo_08_user_research.tex §§8.11.1–8.11.2; archivos fuente del cuestionario/datos por localizar</x:v>
       </x:c>
       <x:c r="N32" s="10" t="str">
-        <x:v>El texto informa 167 respuestas, pero en este repositorio no se localizó un cuestionario ni tabulación por ítem que permita reconstruir elegibilidad, exclusiones y denominadores.</x:v>
+        <x:v>H31: se localizaron imágenes insertadas de resultados de encuesta en images/user_research/fig_08_*.png y su presentación en capítulos; no se localizó exportación de respuestas ni tabla fuente de respuestas individuales. Los porcentajes/figuras no bastan para recomputar denominadores.</x:v>
       </x:c>
       <x:c r="O32" s="10" t="str">
-        <x:v>Solicitar/localizar cuestionario y exportación agregada original; no reconstruir respuestas ni denominadores desde porcentajes del PDF.</x:v>
+        <x:v>Solicitar exportación original de respuestas (CSV/XLSX del formulario) con fecha/campos y versión del cuestionario; si no existe, mantener el bloqueo y no reconstruir respuestas desde las figuras.</x:v>
       </x:c>
       <x:c r="P32" s="10" t="str"/>
       <x:c r="Q32" s="10" t="str">
@@ -3229,10 +3233,10 @@
         <x:v>chapters/capitulo_08_user_research.tex §8.3; appendices/anexo_d_entrevistas.tex D.1–D.5; documentos de consentimiento por localizar</x:v>
       </x:c>
       <x:c r="N46" s="10" t="str">
-        <x:v>Los anexos incluyen nombres, matrículas, referencias profesionales y transcripciones; el paquete no contiene consentimiento ni fechas fuente suficientes para autorizar nuevas afirmaciones o agradecimientos.</x:v>
+        <x:v>H45: el Anexo D aporta transcripciones documentales, no audios originales ni metadatos verificables de sesión.</x:v>
       </x:c>
       <x:c r="O46" s="10" t="str">
-        <x:v>No publicar detalles personales adicionales ni completar consentimientos retroactivamente; localizar autorizaciones existentes y limitar la versión a evidencia autorizada.</x:v>
+        <x:v>Solicitar audio fuente de las entrevistas citadas y registro fechado que permita cotejar la transcripción; adjuntar consentimiento/autorización aplicable.</x:v>
       </x:c>
       <x:c r="P46" s="10" t="str"/>
       <x:c r="Q46" s="10" t="str">
@@ -3862,10 +3866,10 @@
         <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.2; chapters/capitulo_11_capacidades_prototipo.tex §11.11.2; chapters/capitulo_15_modelo_negocio.tex; artifacts/manifests del clasificador subarticular</x:v>
       </x:c>
       <x:c r="N57" s="10" t="str">
-        <x:v>La tesis asocia LumbarDISC/RSNA a un clasificador y proyecta SaaS, pero falta análisis de términos del acuerdo aplicable, cadena de acceso/derivados y relación entre uso académico actual y uso comercial futuro. No se concluye incompatibilidad jurídica con la evidencia disponible.</x:v>
+        <x:v>H56: model cards/manifests registran SPIDER, RSNA/LumbarDISC y hashes de checkpoints/manifests; en el snapshot no se localizaron licencias/terms of use por dataset ni permisos de redistribución/uso comercial para datasets, pesos o checkpoints. Disponibilidad local no acredita derechos comerciales.</x:v>
       </x:c>
       <x:c r="O57" s="10" t="str">
-        <x:v>Mantener bloqueado hasta adjuntar y revisar términos/licencias vigentes por dataset/modelo, alcance de redistribución y uso comercial; documentar límite sin emitir conclusión legal no sustentada.</x:v>
+        <x:v>Solicitar texto de licencia/terms aplicable a cada dataset (SPIDER, RSNA, LumbarDISC), condiciones de los checkpoints/pesos y autorización de redistribución/uso comercial si se pretende.</x:v>
       </x:c>
       <x:c r="P57" s="10" t="str"/>
       <x:c r="Q57" s="10" t="str">
@@ -4269,10 +4273,10 @@
         <x:v>chapters/capitulo_06_estado_del_arte.tex §6.3.3; chapters/capitulo_13_resultados_evaluacion.tex Tabla 13.1; manifests/notebooks axiales</x:v>
       </x:c>
       <x:c r="N64" s="10" t="str">
-        <x:v>515 pacientes y 1.545 máscaras se infieren como 3 niveles por paciente, pero el conteo observado y el universo de evaluación no están reconciliados con 81/102 casos; el paquete no contiene manifest concluyente.</x:v>
+        <x:v>H63: el model card sagital identifica SPIDER, clases agrupadas y hashes; el manifest axial reporta split de prueba bloqueado/opaque sin IDs. No se localizaron máscaras fuente ni paquete de anotaciones con autoría, protocolo y conteos trazables dentro del snapshot. Notebooks procesan máscaras pero no sustituyen su fuente/procedencia.</x:v>
       </x:c>
       <x:c r="O64" s="10" t="str">
-        <x:v>Localizar release exacto, manifest y cuaderno; verificar máscaras y pacientes únicos antes de corregir conteos. No reconstruir cifras por multiplicación sola.</x:v>
+        <x:v>Solicitar paquete fuente de máscaras/etiquetas para cada modelo, manifest de pacientes/estudios asociado y protocolo/registro de etiquetado con autoría y conteos.</x:v>
       </x:c>
       <x:c r="P64" s="10" t="str"/>
       <x:c r="Q64" s="10" t="str">
@@ -4444,10 +4448,10 @@
         <x:v>chapters/capitulo_08_user_research.tex §§8.3–8.4; appendices/anexo_d_entrevistas.tex D.1–D.5</x:v>
       </x:c>
       <x:c r="N67" s="10" t="str">
-        <x:v>Las transcripciones no contienen fechas/duraciones para todas las sesiones; el texto aporta referencias de perfil cuyo soporte no está adjunto. No se puede confirmar consentimiento ni reconstruir metadata.</x:v>
+        <x:v>H66: Anexo D contiene transcripciones documentales; faltan audios originales, fechas de sesión y consentimientos/autorizaciones verificables para publicar atribuciones o perfiles ampliados.</x:v>
       </x:c>
       <x:c r="O67" s="10" t="str">
-        <x:v>Limitar perfiles a datos respaldados por las fuentes disponibles; localizar fechas/consentimientos/autorización antes de publicar información personal adicional.</x:v>
+        <x:v>Solicitar audios originales, agenda/registro fechado y consentimientos/autorizaciones de publicación; conservar atribuciones actuales en el límite que permiten las transcripciones.</x:v>
       </x:c>
       <x:c r="P67" s="10" t="str"/>
       <x:c r="Q67" s="10" t="str">

</xml_diff>

<commit_message>
audit(pfi): record reconciliation commit references
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -1083,7 +1083,7 @@
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
-          <t>0454dc38ce0e12c3267e73b5fcb4b852c3cfde89</t>
+          <t>c7c5490c9ff789463e89993c1a44e5646d702ce3</t>
         </is>
       </c>
       <c r="Q4" s="10" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
-          <t>461cd1a5a7efed8840f7008116e713208cda125a</t>
+          <t>c7c5490c9ff789463e89993c1a44e5646d702ce3</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">

</xml_diff>

<commit_message>
audit(pfi): qualify dataset mask coverage and reproducibility
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -1170,18 +1170,18 @@
       </c>
       <c r="N5" s="10" t="inlineStr">
         <is>
-          <t>H04: el model card sagital publica solo Dice macro no-background 0.8934 e IoU macro 0.8080; no expone los tres Dice por clase. El model card axial sí trae métricas Dice/IoU por clase (raw_0 test Dice 0.1545; raw_50 0.9316; raw_100 0.8400; raw_150 0.7955; raw_200 0.6752). Gate axial no aprobado (macro foreground 0.67935). Evidencia: modelos/final/*.modelcard.md y *.manifest.json del snapshot AI.</t>
+          <t>H04: axial model card trae Dice/IoU por clase y gate fail 0,679348. Sagital model card solo macro Dice 0,8934 / IoU 0,8080. Requisitos para métricas por clase: checkpoint+SHA, split+hash, mapping clase/background, predicciones/GT por caso, protocolo de agregación y script/versionado. No se fabricaron métricas.</t>
         </is>
       </c>
       <c r="O5" s="10" t="inlineStr">
         <is>
-          <t>Completar solo las celdas de métrica que correspondan a cada modelo y dejar explícita la ausencia de desglose por clase para el modelo sagital. No volver a presentar el macro promedio como gate aprobado.</t>
+          <t>Dejar explícita ausencia del desglose sagital hasta recibir artefactos reproducibles; conservar las cifras macro y resultados axiales de fuente.</t>
         </is>
       </c>
       <c r="P5" s="10" t="str"/>
       <c r="Q5" s="10" t="inlineStr">
         <is>
-          <t>No se recalcularon métricas; QA de artefacto pendiente.</t>
+          <t>La compilación no agrega resultados ni altera métricas. pdfLaTeX/Biber/pdfLaTeX/pdfLaTeX exit 0, 232 páginas físicas; sin referencias/citas indefinidas.</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -6501,18 +6501,18 @@
       </c>
       <c r="N64" s="10" t="inlineStr">
         <is>
-          <t>H63: el model card sagital identifica SPIDER, clases agrupadas y hashes; el manifest axial reporta split de prueba bloqueado/opaque sin IDs. No se localizaron máscaras fuente ni paquete de anotaciones con autoría, protocolo y conteos trazables dentro del snapshot. Notebooks procesan máscaras pero no sustituyen su fuente/procedencia.</t>
+          <t>La evidencia del repositorio describe 515 pacientes y procesamiento/uso de etiquetas, pero no aporta paquete fuente completo ni inventario verificable de 1.545 máscaras. Se retiró “cobertura completa”; 515×3 se explica como combinaciones paciente-nivel nominales, no conteo auditado. H63 sigue bloqueado.</t>
         </is>
       </c>
       <c r="O64" s="10" t="inlineStr">
         <is>
-          <t>Solicitar paquete fuente de máscaras/etiquetas para cada modelo, manifest de pacientes/estudios asociado y protocolo/registro de etiquetado con autoría y conteos.</t>
+          <t>Para cerrar: paquete de máscaras/etiquetas, índice por archivo/paciente/nivel, mapping T1→T2, manifest enlazado y protocolo/autoría de anotación; no inferir cobertura desde E9 (610 filas/184 pacientes).</t>
         </is>
       </c>
       <c r="P64" s="10" t="str"/>
       <c r="Q64" s="10" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>PDF físico p.29 reformulado; p.42 FODA matizada por H56/H63. Compilación exit 0; texto extraído confirma desaparición de la afirmación absoluta. Revisión de evidencia, sin auditoría de contenido anatómico de máscaras.</t>
         </is>
       </c>
       <c r="R64" s="10" t="inlineStr">

</xml_diff>

<commit_message>
audit(pfi): record H63 and H04 commit references
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -1178,7 +1178,11 @@
           <t>Dejar explícita ausencia del desglose sagital hasta recibir artefactos reproducibles; conservar las cifras macro y resultados axiales de fuente.</t>
         </is>
       </c>
-      <c r="P5" s="10" t="str"/>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>de37d9cea6ca0c46f0b5878f849723e04eac0789</t>
+        </is>
+      </c>
       <c r="Q5" s="10" t="inlineStr">
         <is>
           <t>La compilación no agrega resultados ni altera métricas. pdfLaTeX/Biber/pdfLaTeX/pdfLaTeX exit 0, 232 páginas físicas; sin referencias/citas indefinidas.</t>
@@ -6509,7 +6513,11 @@
           <t>Para cerrar: paquete de máscaras/etiquetas, índice por archivo/paciente/nivel, mapping T1→T2, manifest enlazado y protocolo/autoría de anotación; no inferir cobertura desde E9 (610 filas/184 pacientes).</t>
         </is>
       </c>
-      <c r="P64" s="10" t="str"/>
+      <c r="P64" s="10" t="inlineStr">
+        <is>
+          <t>de37d9cea6ca0c46f0b5878f849723e04eac0789</t>
+        </is>
+      </c>
       <c r="Q64" s="10" t="inlineStr">
         <is>
           <t>PDF físico p.29 reformulado; p.42 FODA matizada por H56/H63. Compilación exit 0; texto extraído confirma desaparición de la afirmación absoluta. Revisión de evidencia, sin auditoría de contenido anatómico de máscaras.</t>

</xml_diff>

<commit_message>
audit(pfi): define extension scope and acceptance limits
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -1707,12 +1707,12 @@
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>En investigación</t>
+          <t>Cerrado con evidencia</t>
         </is>
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
@@ -1732,18 +1732,18 @@
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t>El capítulo 11 documenta Demo Mode, exportación PDF/JSON, Grad-CAM experimental, 67B2/67C y chat mock/Qwen como capacidades con estados diferenciados. Falta revisar trazabilidad formal a alcance/RF y la frase de exclusión de LLM.</t>
+          <t>Criterio H10: las extensiones no estaban delimitadas formalmente respecto del alcance/RF y “no LLM” podía leerse como exclusión global. §5.5 ahora define Demo Mode/fixtures, exportaciones PDF/JSON, Grad-CAM experimental, 67B2 sin paridad, 67C experimental y chat mock/Qwen no productivo como extensiones sin RF de aceptación del flujo principal; §7/§11 aclaran que solo el preinforme es determinístico por plantillas.</t>
         </is>
       </c>
       <c r="O11" s="10" t="inlineStr">
         <is>
-          <t>Cruzar cada elemento con alcance, RF y código; resolver solo los casos sin definición/estado consistente.</t>
+          <t>§5.5 agregado con referencias cruzadas a estado y evidencia de capacidades. No cambiar flags técnicos ni afirmar Qwen productivo.</t>
         </is>
       </c>
       <c r="P11" s="10" t="str"/>
       <c r="Q11" s="10" t="inlineStr">
         <is>
-          <t>No se modificó el alcance ni se verificó proveedor productivo.</t>
+          <t>QA documental: referencias cruzadas resueltas; pdfLaTeX/Biber/pdfLaTeX/pdfLaTeX exit 0; PDF 233 páginas físicas; revisión visual p.25; sin referencias/citas indefinidas.</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="Q64" s="10" t="inlineStr">
         <is>
-          <t>PDF físico p.29 reformulado; p.42 FODA matizada por H56/H63. Compilación exit 0; texto extraído confirma desaparición de la afirmación absoluta. Revisión de evidencia, sin auditoría de contenido anatómico de máscaras.</t>
+          <t>QA: PDF físico p.29 sin afirmación absoluta; FODA p.43 matizada. PDF final 233 páginas; compilación exit 0 y sin referencias/citas indefinidas. H63 sigue bloqueado por evidencia fuente ausente.</t>
         </is>
       </c>
       <c r="R64" s="10" t="inlineStr">

</xml_diff>

<commit_message>
audit(pfi): link H10 in the master matrix
</commit_message>
<xml_diff>
--- a/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
+++ b/docs/audit/pfi_100_tutor_2026_10_14/MATRIZ_SEGUIMIENTO_AUDITORIA_PFI_100_2026.xlsx
@@ -1740,7 +1740,11 @@
           <t>§5.5 agregado con referencias cruzadas a estado y evidencia de capacidades. No cambiar flags técnicos ni afirmar Qwen productivo.</t>
         </is>
       </c>
-      <c r="P11" s="10" t="str"/>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>b549056f7e56308a977c5e5c618943b72e5a2535</t>
+        </is>
+      </c>
       <c r="Q11" s="10" t="inlineStr">
         <is>
           <t>QA documental: referencias cruzadas resueltas; pdfLaTeX/Biber/pdfLaTeX/pdfLaTeX exit 0; PDF 233 páginas físicas; revisión visual p.25; sin referencias/citas indefinidas.</t>

</xml_diff>